<commit_message>
added archive clearance and just completed all the formats
</commit_message>
<xml_diff>
--- a/uploads/cases.xlsx
+++ b/uploads/cases.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O13"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -859,9 +859,150 @@
         <v>Test Offense 2</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2342323</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Invalid Date</v>
+      </c>
+      <c r="C11" t="str">
+        <v>josshh</v>
+      </c>
+      <c r="D11" t="str">
+        <v>ssds</v>
+      </c>
+      <c r="E11" t="str">
+        <v>loboc</v>
+      </c>
+      <c r="F11" t="str">
+        <v>theft</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Invalid Date</v>
+      </c>
+      <c r="H11" t="str">
+        <v>2026-01-07</v>
+      </c>
+      <c r="I11" t="str">
+        <v>james</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Reppublic Act 2104</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Tagbi</v>
+      </c>
+      <c r="L11" t="str">
+        <v>2026-01-08</v>
+      </c>
+      <c r="M11" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N11" t="str">
+        <v>14k</v>
+      </c>
+      <c r="O11" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>7567564</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Invalid Date</v>
+      </c>
+      <c r="C12" t="str">
+        <v>isabel</v>
+      </c>
+      <c r="D12" t="str">
+        <v>asas</v>
+      </c>
+      <c r="E12" t="str">
+        <v>maribojoc</v>
+      </c>
+      <c r="F12" t="str">
+        <v xml:space="preserve">tax </v>
+      </c>
+      <c r="G12" t="str">
+        <v>Invalid Date</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2026-01-30</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Atty. Superman</v>
+      </c>
+      <c r="J12" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K12" t="str">
+        <v>tagbi</v>
+      </c>
+      <c r="L12" t="str">
+        <v>2026-01-29</v>
+      </c>
+      <c r="M12" t="str">
+        <v>terminated</v>
+      </c>
+      <c r="N12" t="str">
+        <v>12k</v>
+      </c>
+      <c r="O12" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>8678675</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Invalid Date</v>
+      </c>
+      <c r="C13" t="str">
+        <v>mark</v>
+      </c>
+      <c r="D13" t="str">
+        <v>wasdas</v>
+      </c>
+      <c r="E13" t="str">
+        <v>buol</v>
+      </c>
+      <c r="F13" t="str">
+        <v>raped</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Invalid Date</v>
+      </c>
+      <c r="H13" t="str">
+        <v>2026-01-13</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Atty. Doroy</v>
+      </c>
+      <c r="J13" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Capitol</v>
+      </c>
+      <c r="L13" t="str">
+        <v>2026-01-22</v>
+      </c>
+      <c r="M13" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N13" t="str">
+        <v>15k</v>
+      </c>
+      <c r="O13" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added feature for adding MR filed
</commit_message>
<xml_diff>
--- a/uploads/cases.xlsx
+++ b/uploads/cases.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q105"/>
+  <dimension ref="A1:Q110"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -479,37 +479,34 @@
         <v>Invalid Date</v>
       </c>
       <c r="C2" t="str">
-        <v>EVANGELINE M. GABI</v>
+        <v>["EVANGELINE M. GABI"]</v>
       </c>
       <c r="D2" t="str">
-        <v>VII-14-INV 23F-299</v>
+        <v>["VII-14-INV 23F-299"]</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>[""]</v>
       </c>
       <c r="F2" t="str">
         <v>ESTAFA IN REL. TO R.A. 10175 KNOWN AS CYBERCRIME PREVENTION ACT OF 2021</v>
       </c>
-      <c r="H2" t="str">
-        <v>Invalid Date</v>
-      </c>
       <c r="I2" t="str">
         <v>J. R. CESAR</v>
       </c>
       <c r="J2" t="str">
-        <v>R-25552</v>
+        <v>["R-25552"]</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>["2"]</v>
       </c>
       <c r="L2" t="str">
         <v>Invalid Date</v>
       </c>
+      <c r="M2" t="str">
+        <v>[""]</v>
+      </c>
       <c r="N2" t="str">
-        <v/>
-      </c>
-      <c r="O2" t="str">
-        <v/>
+        <v>["Pending"]</v>
       </c>
       <c r="Q2" t="str">
         <v>INDEX CARDS\ABALOS, LUCELLE y TUDTUD_0001.pdf</v>
@@ -4623,43 +4620,40 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>test232</v>
+        <v>VII-14-INQ-22C-134241</v>
       </c>
       <c r="B103" t="str">
-        <v>2026-03-24</v>
+        <v>2026-03-14</v>
       </c>
       <c r="C103" t="str">
-        <v>popo</v>
+        <v>darylss</v>
       </c>
       <c r="D103" t="str">
-        <v>["clemen","sofia","daryl","joshua"]</v>
+        <v>["testt","asda","asd"]</v>
       </c>
       <c r="E103" t="str">
-        <v>san isidro bohol</v>
+        <v>Anda Bohol</v>
       </c>
       <c r="F103" t="str">
-        <v>robbery</v>
-      </c>
-      <c r="H103" t="str">
-        <v>2026-03-25</v>
+        <v>asd</v>
       </c>
       <c r="I103" t="str">
-        <v>atty doroy</v>
+        <v>asdas</v>
       </c>
       <c r="J103" t="str">
-        <v>5675665</v>
+        <v>N/A</v>
       </c>
       <c r="K103" t="str">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="L103" t="str">
+        <v>2026-03-26</v>
       </c>
       <c r="M103" t="str">
-        <v>guilty</v>
+        <v>Ongoing</v>
       </c>
       <c r="N103" t="str">
-        <v>Filed in court</v>
-      </c>
-      <c r="P103" t="str">
-        <v>2026-03-26</v>
+        <v>Convicted</v>
       </c>
       <c r="Q103" t="str">
         <v>N/A</v>
@@ -4673,22 +4667,31 @@
         <v>2026-03-18</v>
       </c>
       <c r="C104" t="str">
-        <v>daryl</v>
+        <v>test</v>
       </c>
       <c r="D104" t="str">
-        <v>["testt"]</v>
+        <v>["test1","test2","test3"]</v>
       </c>
       <c r="E104" t="str">
         <v>Anda Bohol</v>
       </c>
       <c r="F104" t="str">
-        <v>asd</v>
+        <v>attempted murder</v>
+      </c>
+      <c r="H104" t="str">
+        <v>2026-03-26</v>
       </c>
       <c r="I104" t="str">
-        <v>asdas</v>
+        <v>Atty. Joshua</v>
       </c>
       <c r="J104" t="str">
-        <v>N/A</v>
+        <v>4467565</v>
+      </c>
+      <c r="L104" t="str">
+        <v>2026-03-13</v>
+      </c>
+      <c r="M104" t="str">
+        <v>guilty</v>
       </c>
       <c r="N104" t="str">
         <v>Dismissed</v>
@@ -4699,48 +4702,274 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>VII-14-INQ-22C-134241</v>
+        <v>VII-14-INQ-22C-134242</v>
       </c>
       <c r="B105" t="str">
-        <v>2026-03-14</v>
+        <v>2026-03-18</v>
       </c>
       <c r="C105" t="str">
-        <v>darylss</v>
+        <v>kian</v>
       </c>
       <c r="D105" t="str">
-        <v>["testt","asda","asd"]</v>
+        <v>["test14","tes4","test6"]</v>
       </c>
       <c r="E105" t="str">
         <v>Anda Bohol</v>
       </c>
       <c r="F105" t="str">
-        <v>asd</v>
+        <v>attempted murder</v>
+      </c>
+      <c r="H105" t="str">
+        <v>2026-03-26</v>
       </c>
       <c r="I105" t="str">
-        <v>asdas</v>
+        <v>Atty. Joshua</v>
       </c>
       <c r="J105" t="str">
-        <v>N/A</v>
+        <v>635464</v>
       </c>
       <c r="K105" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L105" t="str">
         <v>2026-03-26</v>
       </c>
       <c r="M105" t="str">
-        <v>Ongoing</v>
+        <v>attempted</v>
       </c>
       <c r="N105" t="str">
+        <v>Dismissed</v>
+      </c>
+      <c r="P105" t="str">
+        <v>2026-03-16</v>
+      </c>
+      <c r="Q105" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>VII-14-INQ-22C-13426</v>
+      </c>
+      <c r="B106" t="str">
+        <v>2026-02-07</v>
+      </c>
+      <c r="C106" t="str">
+        <v>John Sotto</v>
+      </c>
+      <c r="D106" t="str">
+        <v>["Vico Sotto"]</v>
+      </c>
+      <c r="E106" t="str">
+        <v>Booy, Tagbilaran City</v>
+      </c>
+      <c r="F106" t="str">
+        <v>Viol. of R.A. 9262 (VAWC)</v>
+      </c>
+      <c r="G106" t="str">
+        <v>2026-02-03</v>
+      </c>
+      <c r="H106" t="str">
+        <v>2026-03-06</v>
+      </c>
+      <c r="I106" t="str">
+        <v>Pros. Doroy</v>
+      </c>
+      <c r="N106" t="str">
+        <v>Dismissed</v>
+      </c>
+      <c r="Q106" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>VII-14-INQ-22C-13423</v>
+      </c>
+      <c r="B107" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="C107" t="str">
+        <v>["aman"]</v>
+      </c>
+      <c r="D107" t="str">
+        <v>["shomin"]</v>
+      </c>
+      <c r="E107" t="str">
+        <v>["testt"]</v>
+      </c>
+      <c r="F107" t="str">
+        <v>murder</v>
+      </c>
+      <c r="G107" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="H107" t="str">
+        <v>2026-03-25</v>
+      </c>
+      <c r="I107" t="str">
+        <v>adolfo foroy</v>
+      </c>
+      <c r="J107" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N107" t="str">
         <v>Convicted</v>
       </c>
-      <c r="Q105" t="str">
-        <v>N/A</v>
+      <c r="P107" t="str">
+        <v>2026-03-17</v>
+      </c>
+      <c r="Q107" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>VII-345-67567</v>
+      </c>
+      <c r="B108" t="str">
+        <v>2026-03-25</v>
+      </c>
+      <c r="C108" t="str">
+        <v>["kopiko","totong","sosoy"]</v>
+      </c>
+      <c r="D108" t="str">
+        <v>["Compuesto","Test 3","juancho"]</v>
+      </c>
+      <c r="E108" t="str">
+        <v>["calape","tubigon","sagbayan"]</v>
+      </c>
+      <c r="F108" t="str">
+        <v>murder</v>
+      </c>
+      <c r="H108" t="str">
+        <v>2026-03-17</v>
+      </c>
+      <c r="I108" t="str">
+        <v>Atty. Joshua</v>
+      </c>
+      <c r="J108" t="str">
+        <v>657453</v>
+      </c>
+      <c r="K108" t="str">
+        <v>2</v>
+      </c>
+      <c r="L108" t="str">
+        <v>2026-03-23</v>
+      </c>
+      <c r="M108" t="str">
+        <v>Robbery</v>
+      </c>
+      <c r="N108" t="str">
+        <v>Dismissed</v>
+      </c>
+      <c r="P108" t="str">
+        <v>2026-03-22</v>
+      </c>
+      <c r="Q108" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>VII-14-INQ-23H-195</v>
+      </c>
+      <c r="B109" t="str">
+        <v>2023-07-29</v>
+      </c>
+      <c r="C109" t="str">
+        <v>["PNP-TAGBILARAN CITY"]</v>
+      </c>
+      <c r="D109" t="str">
+        <v>["ZAIMON ABAY y LUMAGBAS","JOSEPH LIM III y ZAFRA"]</v>
+      </c>
+      <c r="E109" t="str">
+        <v>["Tagbilaran City","Tagbilaran City"]</v>
+      </c>
+      <c r="F109" t="str">
+        <v>Violation of Sec. 5, Art. II of R.A. 9165</v>
+      </c>
+      <c r="H109" t="str">
+        <v>2023-07-29</v>
+      </c>
+      <c r="I109" t="str">
+        <v>Josie Vida C. Sempron</v>
+      </c>
+      <c r="J109" t="str">
+        <v>["R-27679","R-27679"]</v>
+      </c>
+      <c r="K109" t="str">
+        <v>["4","1"]</v>
+      </c>
+      <c r="L109" t="str">
+        <v>Invalid Date</v>
+      </c>
+      <c r="M109" t="str">
+        <v>["murder","robbery"]</v>
+      </c>
+      <c r="N109" t="str">
+        <v>["Filed in Court","Filed in Court"]</v>
+      </c>
+      <c r="P109" t="str">
+        <v>2026-03-09</v>
+      </c>
+      <c r="Q109" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>VII-14-INQ-22C-13424175</v>
+      </c>
+      <c r="B110" t="str">
+        <v>2026-02-21</v>
+      </c>
+      <c r="C110" t="str">
+        <v>["jep2","mimimng","dodong"]</v>
+      </c>
+      <c r="D110" t="str">
+        <v>["simba","totong","jopay kamusta kana"]</v>
+      </c>
+      <c r="E110" t="str">
+        <v>["taloto","koroko"]</v>
+      </c>
+      <c r="F110" t="str">
+        <v>murder</v>
+      </c>
+      <c r="G110" t="str">
+        <v>2026-02-14</v>
+      </c>
+      <c r="H110" t="str">
+        <v>2026-02-20</v>
+      </c>
+      <c r="I110" t="str">
+        <v>Atty. Doroy</v>
+      </c>
+      <c r="J110" t="str">
+        <v>["N/A","N/A","4534543"]</v>
+      </c>
+      <c r="K110" t="str">
+        <v>["2","2","2"]</v>
+      </c>
+      <c r="L110" t="str">
+        <v>Invalid Date</v>
+      </c>
+      <c r="M110" t="str">
+        <v>["","","attempted"]</v>
+      </c>
+      <c r="N110" t="str">
+        <v>["Dismissed","Dismissed","Filed in Court"]</v>
+      </c>
+      <c r="P110" t="str">
+        <v>2026-02-20</v>
+      </c>
+      <c r="Q110" t="str">
+        <v>/uploads/index_cards/indexcard-1773238533278-115631718.png</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q105"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q110"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Mr filed respondent and the decision each of te respondent
</commit_message>
<xml_diff>
--- a/uploads/cases.xlsx
+++ b/uploads/cases.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q110"/>
+  <dimension ref="A1:Q104"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4620,40 +4620,46 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>VII-14-INQ-22C-134241</v>
+        <v>VII-14-INQ-23H-195</v>
       </c>
       <c r="B103" t="str">
-        <v>2026-03-14</v>
+        <v>2023-07-29</v>
       </c>
       <c r="C103" t="str">
-        <v>darylss</v>
+        <v>["PNP-TAGBILARAN CITY"]</v>
       </c>
       <c r="D103" t="str">
-        <v>["testt","asda","asd"]</v>
+        <v>["ZAIMON ABAY y LUMAGBAS","JOSEPH LIM III y ZAFRA"]</v>
       </c>
       <c r="E103" t="str">
-        <v>Anda Bohol</v>
+        <v>["Tagbilaran City","Tagbilaran City"]</v>
       </c>
       <c r="F103" t="str">
-        <v>asd</v>
+        <v>Violation of Sec. 5, Art. II of R.A. 9165</v>
+      </c>
+      <c r="H103" t="str">
+        <v>2023-07-29</v>
       </c>
       <c r="I103" t="str">
-        <v>asdas</v>
+        <v>Josie Vida C. Sempron</v>
       </c>
       <c r="J103" t="str">
-        <v>N/A</v>
+        <v>["R-27679","R-27679"]</v>
       </c>
       <c r="K103" t="str">
-        <v>3</v>
+        <v>["4","1"]</v>
       </c>
       <c r="L103" t="str">
-        <v>2026-03-26</v>
+        <v>Invalid Date</v>
       </c>
       <c r="M103" t="str">
-        <v>Ongoing</v>
+        <v>["murder","robbery"]</v>
       </c>
       <c r="N103" t="str">
-        <v>Convicted</v>
+        <v>["Filed in Court","Filed in Court"]</v>
+      </c>
+      <c r="P103" t="str">
+        <v>2026-03-09</v>
       </c>
       <c r="Q103" t="str">
         <v>N/A</v>
@@ -4661,315 +4667,57 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>VII-14-INQ-22C-13424</v>
+        <v>Test_2123</v>
       </c>
       <c r="B104" t="str">
-        <v>2026-03-18</v>
+        <v>2026-03-16</v>
       </c>
       <c r="C104" t="str">
-        <v>test</v>
+        <v>["Kian Bullanday","Rainer Goloso","Ken Maniwang"]</v>
       </c>
       <c r="D104" t="str">
-        <v>["test1","test2","test3"]</v>
+        <v>["James Lloyd Antiola","Joshua Galamiton","Jeff Alexis Arcayan"]</v>
       </c>
       <c r="E104" t="str">
-        <v>Anda Bohol</v>
+        <v>["San Isidro Bohol","Jagna Bohol","Tagbilaran Bohol"]</v>
       </c>
       <c r="F104" t="str">
-        <v>attempted murder</v>
+        <v>Attempted Murder</v>
       </c>
       <c r="H104" t="str">
-        <v>2026-03-26</v>
+        <v>2026-03-15</v>
       </c>
       <c r="I104" t="str">
-        <v>Atty. Joshua</v>
+        <v xml:space="preserve">Atty.Arvin </v>
       </c>
       <c r="J104" t="str">
-        <v>4467565</v>
+        <v>["23434534","45634523423","56234"]</v>
+      </c>
+      <c r="K104" t="str">
+        <v>["3","1","1"]</v>
       </c>
       <c r="L104" t="str">
-        <v>2026-03-13</v>
+        <v>Invalid Date</v>
       </c>
       <c r="M104" t="str">
-        <v>guilty</v>
+        <v>["murder","attempted murder","robbery"]</v>
       </c>
       <c r="N104" t="str">
-        <v>Dismissed</v>
+        <v>["Filed in Court","Filed in Court","Filed in Court"]</v>
+      </c>
+      <c r="O104" t="str">
+        <v>community service</v>
+      </c>
+      <c r="P104" t="str">
+        <v>2026-03-29</v>
       </c>
       <c r="Q104" t="str">
         <v>N/A</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="str">
-        <v>VII-14-INQ-22C-134242</v>
-      </c>
-      <c r="B105" t="str">
-        <v>2026-03-18</v>
-      </c>
-      <c r="C105" t="str">
-        <v>kian</v>
-      </c>
-      <c r="D105" t="str">
-        <v>["test14","tes4","test6"]</v>
-      </c>
-      <c r="E105" t="str">
-        <v>Anda Bohol</v>
-      </c>
-      <c r="F105" t="str">
-        <v>attempted murder</v>
-      </c>
-      <c r="H105" t="str">
-        <v>2026-03-26</v>
-      </c>
-      <c r="I105" t="str">
-        <v>Atty. Joshua</v>
-      </c>
-      <c r="J105" t="str">
-        <v>635464</v>
-      </c>
-      <c r="K105" t="str">
-        <v>2</v>
-      </c>
-      <c r="L105" t="str">
-        <v>2026-03-26</v>
-      </c>
-      <c r="M105" t="str">
-        <v>attempted</v>
-      </c>
-      <c r="N105" t="str">
-        <v>Dismissed</v>
-      </c>
-      <c r="P105" t="str">
-        <v>2026-03-16</v>
-      </c>
-      <c r="Q105" t="str">
-        <v>N/A</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="str">
-        <v>VII-14-INQ-22C-13426</v>
-      </c>
-      <c r="B106" t="str">
-        <v>2026-02-07</v>
-      </c>
-      <c r="C106" t="str">
-        <v>John Sotto</v>
-      </c>
-      <c r="D106" t="str">
-        <v>["Vico Sotto"]</v>
-      </c>
-      <c r="E106" t="str">
-        <v>Booy, Tagbilaran City</v>
-      </c>
-      <c r="F106" t="str">
-        <v>Viol. of R.A. 9262 (VAWC)</v>
-      </c>
-      <c r="G106" t="str">
-        <v>2026-02-03</v>
-      </c>
-      <c r="H106" t="str">
-        <v>2026-03-06</v>
-      </c>
-      <c r="I106" t="str">
-        <v>Pros. Doroy</v>
-      </c>
-      <c r="N106" t="str">
-        <v>Dismissed</v>
-      </c>
-      <c r="Q106" t="str">
-        <v>N/A</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="str">
-        <v>VII-14-INQ-22C-13423</v>
-      </c>
-      <c r="B107" t="str">
-        <v>2026-03-11</v>
-      </c>
-      <c r="C107" t="str">
-        <v>["aman"]</v>
-      </c>
-      <c r="D107" t="str">
-        <v>["shomin"]</v>
-      </c>
-      <c r="E107" t="str">
-        <v>["testt"]</v>
-      </c>
-      <c r="F107" t="str">
-        <v>murder</v>
-      </c>
-      <c r="G107" t="str">
-        <v>2026-03-10</v>
-      </c>
-      <c r="H107" t="str">
-        <v>2026-03-25</v>
-      </c>
-      <c r="I107" t="str">
-        <v>adolfo foroy</v>
-      </c>
-      <c r="J107" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="N107" t="str">
-        <v>Convicted</v>
-      </c>
-      <c r="P107" t="str">
-        <v>2026-03-17</v>
-      </c>
-      <c r="Q107" t="str">
-        <v>N/A</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="str">
-        <v>VII-345-67567</v>
-      </c>
-      <c r="B108" t="str">
-        <v>2026-03-25</v>
-      </c>
-      <c r="C108" t="str">
-        <v>["kopiko","totong","sosoy"]</v>
-      </c>
-      <c r="D108" t="str">
-        <v>["Compuesto","Test 3","juancho"]</v>
-      </c>
-      <c r="E108" t="str">
-        <v>["calape","tubigon","sagbayan"]</v>
-      </c>
-      <c r="F108" t="str">
-        <v>murder</v>
-      </c>
-      <c r="H108" t="str">
-        <v>2026-03-17</v>
-      </c>
-      <c r="I108" t="str">
-        <v>Atty. Joshua</v>
-      </c>
-      <c r="J108" t="str">
-        <v>657453</v>
-      </c>
-      <c r="K108" t="str">
-        <v>2</v>
-      </c>
-      <c r="L108" t="str">
-        <v>2026-03-23</v>
-      </c>
-      <c r="M108" t="str">
-        <v>Robbery</v>
-      </c>
-      <c r="N108" t="str">
-        <v>Dismissed</v>
-      </c>
-      <c r="P108" t="str">
-        <v>2026-03-22</v>
-      </c>
-      <c r="Q108" t="str">
-        <v>N/A</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="str">
-        <v>VII-14-INQ-23H-195</v>
-      </c>
-      <c r="B109" t="str">
-        <v>2023-07-29</v>
-      </c>
-      <c r="C109" t="str">
-        <v>["PNP-TAGBILARAN CITY"]</v>
-      </c>
-      <c r="D109" t="str">
-        <v>["ZAIMON ABAY y LUMAGBAS","JOSEPH LIM III y ZAFRA"]</v>
-      </c>
-      <c r="E109" t="str">
-        <v>["Tagbilaran City","Tagbilaran City"]</v>
-      </c>
-      <c r="F109" t="str">
-        <v>Violation of Sec. 5, Art. II of R.A. 9165</v>
-      </c>
-      <c r="H109" t="str">
-        <v>2023-07-29</v>
-      </c>
-      <c r="I109" t="str">
-        <v>Josie Vida C. Sempron</v>
-      </c>
-      <c r="J109" t="str">
-        <v>["R-27679","R-27679"]</v>
-      </c>
-      <c r="K109" t="str">
-        <v>["4","1"]</v>
-      </c>
-      <c r="L109" t="str">
-        <v>Invalid Date</v>
-      </c>
-      <c r="M109" t="str">
-        <v>["murder","robbery"]</v>
-      </c>
-      <c r="N109" t="str">
-        <v>["Filed in Court","Filed in Court"]</v>
-      </c>
-      <c r="P109" t="str">
-        <v>2026-03-09</v>
-      </c>
-      <c r="Q109" t="str">
-        <v>N/A</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="str">
-        <v>VII-14-INQ-22C-13424175</v>
-      </c>
-      <c r="B110" t="str">
-        <v>2026-02-21</v>
-      </c>
-      <c r="C110" t="str">
-        <v>["jep2","mimimng","dodong"]</v>
-      </c>
-      <c r="D110" t="str">
-        <v>["simba","totong","jopay kamusta kana"]</v>
-      </c>
-      <c r="E110" t="str">
-        <v>["taloto","koroko"]</v>
-      </c>
-      <c r="F110" t="str">
-        <v>murder</v>
-      </c>
-      <c r="G110" t="str">
-        <v>2026-02-14</v>
-      </c>
-      <c r="H110" t="str">
-        <v>2026-02-20</v>
-      </c>
-      <c r="I110" t="str">
-        <v>Atty. Doroy</v>
-      </c>
-      <c r="J110" t="str">
-        <v>["N/A","N/A","4534543"]</v>
-      </c>
-      <c r="K110" t="str">
-        <v>["2","2","2"]</v>
-      </c>
-      <c r="L110" t="str">
-        <v>Invalid Date</v>
-      </c>
-      <c r="M110" t="str">
-        <v>["","","attempted"]</v>
-      </c>
-      <c r="N110" t="str">
-        <v>["Dismissed","Dismissed","Filed in Court"]</v>
-      </c>
-      <c r="P110" t="str">
-        <v>2026-02-20</v>
-      </c>
-      <c r="Q110" t="str">
-        <v>/uploads/index_cards/indexcard-1773238533278-115631718.png</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q110"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q104"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
counting of cases fixed
</commit_message>
<xml_diff>
--- a/uploads/cases.xlsx
+++ b/uploads/cases.xlsx
@@ -500,7 +500,7 @@
         <v>VII-14-INQ-20I-361</v>
       </c>
       <c r="B2" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C2" t="str">
         <v>TAGBILARAN CITY PNP</v>
@@ -562,7 +562,7 @@
         <v>VII-14-INQ-20I-360</v>
       </c>
       <c r="B3" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C3" t="str">
         <v>TAGBILARAN CITY PNP</v>
@@ -934,7 +934,7 @@
         <v>2005-19</v>
       </c>
       <c r="B9" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C9" t="str">
         <v/>
@@ -996,7 +996,7 @@
         <v>2006-45</v>
       </c>
       <c r="B10" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C10" t="str">
         <v/>
@@ -1120,7 +1120,7 @@
         <v>VII-14-INQ-20A-04</v>
       </c>
       <c r="B12" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C12" t="str">
         <v>SALARDA, MYRA A.</v>
@@ -1306,7 +1306,7 @@
         <v>96-3427-3429</v>
       </c>
       <c r="B15" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C15" t="str">
         <v/>
@@ -1430,7 +1430,7 @@
         <v>3434</v>
       </c>
       <c r="B17" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C17" t="str">
         <v/>
@@ -2050,7 +2050,7 @@
         <v>VII-14-INV-22D-071</v>
       </c>
       <c r="B27" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C27" t="str">
         <v>CIDG-BOHOL</v>
@@ -2112,7 +2112,7 @@
         <v>VII-14-INV-22D-070</v>
       </c>
       <c r="B28" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C28" t="str">
         <v>CIDG-BOHOL</v>
@@ -2174,7 +2174,7 @@
         <v>VII-14-INQ-17A-027</v>
       </c>
       <c r="B29" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C29" t="str">
         <v/>
@@ -2360,7 +2360,7 @@
         <v>24H-260</v>
       </c>
       <c r="B32" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C32" t="str">
         <v>CADAYDAY, NEMESIA</v>
@@ -2422,7 +2422,7 @@
         <v>24H-260</v>
       </c>
       <c r="B33" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C33" t="str">
         <v>CADAYDAY,NEMESIA</v>
@@ -2484,7 +2484,7 @@
         <v>24H-261</v>
       </c>
       <c r="B34" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C34" t="str">
         <v>ALIVIADO, KHY</v>
@@ -2546,7 +2546,7 @@
         <v>24H-261</v>
       </c>
       <c r="B35" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C35" t="str">
         <v>CADAYDAY,NEMESIA</v>
@@ -2608,7 +2608,7 @@
         <v>96-228</v>
       </c>
       <c r="B36" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C36" t="str">
         <v/>
@@ -2670,7 +2670,7 @@
         <v>96-229</v>
       </c>
       <c r="B37" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C37" t="str">
         <v/>
@@ -2732,7 +2732,7 @@
         <v>96-230</v>
       </c>
       <c r="B38" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C38" t="str">
         <v/>
@@ -2794,7 +2794,7 @@
         <v>VII-14-INV-2OL-366</v>
       </c>
       <c r="B39" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C39" t="str">
         <v>PNP - TAGBILARAN CITY</v>
@@ -2980,7 +2980,7 @@
         <v>96-306</v>
       </c>
       <c r="B42" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C42" t="str">
         <v/>
@@ -3042,7 +3042,7 @@
         <v>96-307</v>
       </c>
       <c r="B43" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C43" t="str">
         <v/>
@@ -3104,7 +3104,7 @@
         <v>96-308</v>
       </c>
       <c r="B44" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C44" t="str">
         <v/>
@@ -3352,7 +3352,7 @@
         <v>VII-14-INQ-221-197</v>
       </c>
       <c r="B48" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C48" t="str">
         <v>PDEA-BOHOL</v>
@@ -3476,7 +3476,7 @@
         <v>VII-14-INQ-221-196</v>
       </c>
       <c r="B50" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C50" t="str">
         <v>PDEA-BOHOL</v>
@@ -3538,7 +3538,7 @@
         <v>3145</v>
       </c>
       <c r="B51" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C51" t="str">
         <v/>
@@ -3600,7 +3600,7 @@
         <v>3144</v>
       </c>
       <c r="B52" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C52" t="str">
         <v/>
@@ -3786,7 +3786,7 @@
         <v>VII-14-INV-175-0325</v>
       </c>
       <c r="B55" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C55" t="str">
         <v/>
@@ -3972,7 +3972,7 @@
         <v>VII-14-INV-20A-27</v>
       </c>
       <c r="B58" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C58" t="str">
         <v>CIDG-BOHOL</v>
@@ -4034,7 +4034,7 @@
         <v>VII-14-INV-20A-26</v>
       </c>
       <c r="B59" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C59" t="str">
         <v>CIDG-BOHOL</v>
@@ -4158,7 +4158,7 @@
         <v>2000-129</v>
       </c>
       <c r="B61" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C61" t="str">
         <v/>
@@ -4220,7 +4220,7 @@
         <v>2000-130</v>
       </c>
       <c r="B62" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C62" t="str">
         <v/>
@@ -4282,7 +4282,7 @@
         <v>2000-131</v>
       </c>
       <c r="B63" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C63" t="str">
         <v/>
@@ -4344,7 +4344,7 @@
         <v>2000-132</v>
       </c>
       <c r="B64" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C64" t="str">
         <v/>
@@ -4406,7 +4406,7 @@
         <v>2000-133</v>
       </c>
       <c r="B65" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C65" t="str">
         <v/>
@@ -4468,7 +4468,7 @@
         <v>2000-134</v>
       </c>
       <c r="B66" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C66" t="str">
         <v/>
@@ -4530,7 +4530,7 @@
         <v>2000-135</v>
       </c>
       <c r="B67" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C67" t="str">
         <v/>
@@ -4592,7 +4592,7 @@
         <v>2000-136</v>
       </c>
       <c r="B68" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C68" t="str">
         <v/>
@@ -4654,7 +4654,7 @@
         <v>2000-137</v>
       </c>
       <c r="B69" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C69" t="str">
         <v/>
@@ -4716,7 +4716,7 @@
         <v>2000-138</v>
       </c>
       <c r="B70" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C70" t="str">
         <v/>
@@ -4778,7 +4778,7 @@
         <v>2000-139</v>
       </c>
       <c r="B71" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C71" t="str">
         <v/>
@@ -4840,7 +4840,7 @@
         <v>VII-14-INQ-24K-285</v>
       </c>
       <c r="B72" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C72" t="str">
         <v>NBI-CEBU OFFICE -MANDAUE CITY</v>
@@ -4902,7 +4902,7 @@
         <v>99-317</v>
       </c>
       <c r="B73" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C73" t="str">
         <v/>
@@ -4964,7 +4964,7 @@
         <v>VII-14-INV-20H-207</v>
       </c>
       <c r="B74" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C74" t="str">
         <v>BINAMIRA, GARRY NOEL E.</v>
@@ -5026,7 +5026,7 @@
         <v>24J-242</v>
       </c>
       <c r="B75" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C75" t="str">
         <v>PDEA-BOHOL</v>
@@ -5088,7 +5088,7 @@
         <v>24J-243</v>
       </c>
       <c r="B76" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C76" t="str">
         <v>PDEA-BOHOL</v>
@@ -5150,7 +5150,7 @@
         <v>24J-244</v>
       </c>
       <c r="B77" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C77" t="str">
         <v>PDEA-BOHOL</v>
@@ -5212,7 +5212,7 @@
         <v>24J-245</v>
       </c>
       <c r="B78" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C78" t="str">
         <v>PDEA-BOHOL</v>
@@ -5336,7 +5336,7 @@
         <v>89-289 89-289-A 89-289-B 89-289-C 89-289-D</v>
       </c>
       <c r="B80" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C80" t="str">
         <v/>
@@ -5398,7 +5398,7 @@
         <v>VII-14-INV-21A-079</v>
       </c>
       <c r="B81" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C81" t="str">
         <v>STARLITE MARINE INDUSTRIAL SERVICES CORP.</v>
@@ -5460,7 +5460,7 @@
         <v>24K-300</v>
       </c>
       <c r="B82" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C82" t="str">
         <v>PNP - TAGBILARAN CITY</v>
@@ -6452,7 +6452,7 @@
         <v>96-1464</v>
       </c>
       <c r="B98" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C98" t="str">
         <v/>
@@ -6700,7 +6700,7 @@
         <v>92-195</v>
       </c>
       <c r="B102" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C102" t="str">
         <v/>
@@ -6762,7 +6762,7 @@
         <v>VII-14-INV-24B-55</v>
       </c>
       <c r="B103" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C103" t="str">
         <v>BAJA, NOEL B.</v>
@@ -6824,7 +6824,7 @@
         <v>86-226</v>
       </c>
       <c r="B104" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C104" t="str">
         <v/>
@@ -6886,7 +6886,7 @@
         <v>97-3828</v>
       </c>
       <c r="B105" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C105" t="str">
         <v/>
@@ -6948,7 +6948,7 @@
         <v>97-3829</v>
       </c>
       <c r="B106" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C106" t="str">
         <v/>
@@ -7010,7 +7010,7 @@
         <v>97-3830</v>
       </c>
       <c r="B107" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C107" t="str">
         <v/>
@@ -7072,7 +7072,7 @@
         <v>97-3831</v>
       </c>
       <c r="B108" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C108" t="str">
         <v/>
@@ -7754,7 +7754,7 @@
         <v>3510</v>
       </c>
       <c r="B119" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C119" t="str">
         <v/>
@@ -7816,7 +7816,7 @@
         <v>96-2673</v>
       </c>
       <c r="B120" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C120" t="str">
         <v/>
@@ -7878,7 +7878,7 @@
         <v>96-2674</v>
       </c>
       <c r="B121" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C121" t="str">
         <v/>
@@ -7940,7 +7940,7 @@
         <v>96-2675</v>
       </c>
       <c r="B122" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C122" t="str">
         <v/>
@@ -8002,7 +8002,7 @@
         <v>97-3037</v>
       </c>
       <c r="B123" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C123" t="str">
         <v/>
@@ -8064,7 +8064,7 @@
         <v>97-3038</v>
       </c>
       <c r="B124" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C124" t="str">
         <v/>
@@ -8126,7 +8126,7 @@
         <v>97-3039</v>
       </c>
       <c r="B125" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C125" t="str">
         <v/>
@@ -8188,7 +8188,7 @@
         <v>97-1336</v>
       </c>
       <c r="B126" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C126" t="str">
         <v/>
@@ -8250,7 +8250,7 @@
         <v>97-1336</v>
       </c>
       <c r="B127" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C127" t="str">
         <v/>
@@ -8374,7 +8374,7 @@
         <v>97-1339</v>
       </c>
       <c r="B129" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C129" t="str">
         <v/>
@@ -8436,7 +8436,7 @@
         <v>97-1340</v>
       </c>
       <c r="B130" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C130" t="str">
         <v/>
@@ -8498,7 +8498,7 @@
         <v>97-1341</v>
       </c>
       <c r="B131" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C131" t="str">
         <v/>
@@ -8560,7 +8560,7 @@
         <v>96-2554</v>
       </c>
       <c r="B132" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C132" t="str">
         <v/>
@@ -8622,7 +8622,7 @@
         <v>96-2555</v>
       </c>
       <c r="B133" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C133" t="str">
         <v/>
@@ -8684,7 +8684,7 @@
         <v>96-2556</v>
       </c>
       <c r="B134" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C134" t="str">
         <v/>
@@ -8746,7 +8746,7 @@
         <v>96-2557</v>
       </c>
       <c r="B135" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C135" t="str">
         <v/>
@@ -8808,7 +8808,7 @@
         <v>96-2558</v>
       </c>
       <c r="B136" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C136" t="str">
         <v/>
@@ -8870,7 +8870,7 @@
         <v>24l-222</v>
       </c>
       <c r="B137" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C137" t="str">
         <v>TAGBILARAN CITY - PNP</v>
@@ -8932,7 +8932,7 @@
         <v>24l-223</v>
       </c>
       <c r="B138" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C138" t="str">
         <v>TAGBILARAN CITY - PNP</v>
@@ -9366,7 +9366,7 @@
         <v>97-397</v>
       </c>
       <c r="B145" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C145" t="str">
         <v/>
@@ -9428,7 +9428,7 @@
         <v>2005-537</v>
       </c>
       <c r="B146" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C146" t="str">
         <v/>
@@ -9738,7 +9738,7 @@
         <v>2002-999</v>
       </c>
       <c r="B151" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C151" t="str">
         <v/>
@@ -9800,7 +9800,7 @@
         <v>2002-1000</v>
       </c>
       <c r="B152" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C152" t="str">
         <v/>
@@ -9862,7 +9862,7 @@
         <v>2002-1001</v>
       </c>
       <c r="B153" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C153" t="str">
         <v/>
@@ -9924,7 +9924,7 @@
         <v>2002-1002</v>
       </c>
       <c r="B154" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C154" t="str">
         <v/>
@@ -9986,7 +9986,7 @@
         <v>3961</v>
       </c>
       <c r="B155" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C155" t="str">
         <v/>
@@ -10048,7 +10048,7 @@
         <v>VII-14-INQ-23B-061</v>
       </c>
       <c r="B156" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C156" t="str">
         <v>PIU-BOHOL PPO</v>
@@ -10110,7 +10110,7 @@
         <v>VII-14-INQ-23B-061</v>
       </c>
       <c r="B157" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C157" t="str">
         <v>PIU BOHOL PPO</v>
@@ -10172,7 +10172,7 @@
         <v>VII-14-INQ-23B-062</v>
       </c>
       <c r="B158" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C158" t="str">
         <v>PIU-BOHOL PPO</v>
@@ -10234,7 +10234,7 @@
         <v>VII-14-INQ-23B-062</v>
       </c>
       <c r="B159" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C159" t="str">
         <v>PIU BOHOL PPO</v>
@@ -10420,7 +10420,7 @@
         <v>93-463</v>
       </c>
       <c r="B162" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C162" t="str">
         <v/>
@@ -10482,7 +10482,7 @@
         <v>93-464</v>
       </c>
       <c r="B163" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C163" t="str">
         <v/>
@@ -10544,7 +10544,7 @@
         <v>96-1680</v>
       </c>
       <c r="B164" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C164" t="str">
         <v/>
@@ -10606,7 +10606,7 @@
         <v>96-1681</v>
       </c>
       <c r="B165" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C165" t="str">
         <v/>
@@ -10668,7 +10668,7 @@
         <v>96-1682</v>
       </c>
       <c r="B166" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C166" t="str">
         <v/>
@@ -10730,7 +10730,7 @@
         <v>96-1697</v>
       </c>
       <c r="B167" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C167" t="str">
         <v/>
@@ -10792,7 +10792,7 @@
         <v>96-1698</v>
       </c>
       <c r="B168" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C168" t="str">
         <v/>
@@ -10854,7 +10854,7 @@
         <v>96-1699</v>
       </c>
       <c r="B169" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C169" t="str">
         <v/>
@@ -10978,7 +10978,7 @@
         <v>VII-14-INQ-24J-257</v>
       </c>
       <c r="B171" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C171" t="str">
         <v>PNP-TAGBILARAN CITY</v>
@@ -11040,7 +11040,7 @@
         <v>VII-14-INQ-24J-257</v>
       </c>
       <c r="B172" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C172" t="str">
         <v>PNP- TAGBILARAN CITY</v>
@@ -11102,7 +11102,7 @@
         <v>96-831</v>
       </c>
       <c r="B173" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C173" t="str">
         <v/>
@@ -11164,7 +11164,7 @@
         <v>VII-14-INV-24J-316</v>
       </c>
       <c r="B174" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C174" t="str">
         <v>ROSALEJOS, ALFONSO LIGO</v>
@@ -11226,7 +11226,7 @@
         <v>VII-14-INV-24J-316 b</v>
       </c>
       <c r="B175" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C175" t="str">
         <v>ROSALEJOS, ALFONSO LIGO</v>
@@ -11288,7 +11288,7 @@
         <v>97-3034</v>
       </c>
       <c r="B176" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C176" t="str">
         <v/>
@@ -11350,7 +11350,7 @@
         <v>97-3035</v>
       </c>
       <c r="B177" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C177" t="str">
         <v/>
@@ -11412,7 +11412,7 @@
         <v>97-3036</v>
       </c>
       <c r="B178" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C178" t="str">
         <v/>
@@ -11474,7 +11474,7 @@
         <v>96-1724</v>
       </c>
       <c r="B179" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C179" t="str">
         <v/>
@@ -11536,7 +11536,7 @@
         <v>96-1725</v>
       </c>
       <c r="B180" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C180" t="str">
         <v/>
@@ -11598,7 +11598,7 @@
         <v>96-1726</v>
       </c>
       <c r="B181" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C181" t="str">
         <v/>
@@ -11660,7 +11660,7 @@
         <v>96-1574</v>
       </c>
       <c r="B182" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C182" t="str">
         <v/>
@@ -11722,7 +11722,7 @@
         <v>96-1575</v>
       </c>
       <c r="B183" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C183" t="str">
         <v/>
@@ -11784,7 +11784,7 @@
         <v>96-1576</v>
       </c>
       <c r="B184" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C184" t="str">
         <v/>
@@ -11846,7 +11846,7 @@
         <v>98-004</v>
       </c>
       <c r="B185" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C185" t="str">
         <v/>
@@ -11908,7 +11908,7 @@
         <v>98-005</v>
       </c>
       <c r="B186" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C186" t="str">
         <v/>
@@ -12280,7 +12280,7 @@
         <v>VII-14-INQ-20K-408</v>
       </c>
       <c r="B192" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C192" t="str">
         <v>PNP-TAGBILARAN CITY</v>
@@ -12342,7 +12342,7 @@
         <v>VII-14-INQ-20K-408</v>
       </c>
       <c r="B193" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C193" t="str">
         <v>PNP TAGBILARAN CITY</v>
@@ -12466,7 +12466,7 @@
         <v>VII-14-INQ-19E-197</v>
       </c>
       <c r="B195" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C195" t="str">
         <v>TAGBILARAN CITY POLICE</v>
@@ -13396,7 +13396,7 @@
         <v>VII-14-INV-20E-99</v>
       </c>
       <c r="B210" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C210" t="str">
         <v>FERNANDEZ, EULALIA A.</v>
@@ -13458,7 +13458,7 @@
         <v>VII-14-INV-18D-0132</v>
       </c>
       <c r="B211" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C211" t="str">
         <v>FCB, REP BY: GALAB, ANTHONY B.</v>
@@ -13520,7 +13520,7 @@
         <v>VII-14-INV-17H-0230</v>
       </c>
       <c r="B212" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C212" t="str">
         <v>A-1-BY TAGASLING, JOSEPHINE B.</v>
@@ -13582,7 +13582,7 @@
         <v>VII-14-INV-17H-0230 -A</v>
       </c>
       <c r="B213" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C213" t="str">
         <v>A-1-BY TAGASLING, JOSEPHINE B.</v>
@@ -13644,7 +13644,7 @@
         <v>VII-14-INV-18K-445</v>
       </c>
       <c r="B214" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C214" t="str">
         <v>GALLA, JOHN S.</v>
@@ -13706,7 +13706,7 @@
         <v>VII-14-INV-20E-100</v>
       </c>
       <c r="B215" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C215" t="str">
         <v>FERNANDEZ, EULALIA A.</v>
@@ -13768,7 +13768,7 @@
         <v>VII-14-INV-21B-30</v>
       </c>
       <c r="B216" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C216" t="str">
         <v>CIDG-BOHOL</v>
@@ -13830,7 +13830,7 @@
         <v>VII-14-INV-21B-31</v>
       </c>
       <c r="B217" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C217" t="str">
         <v>CIDG-BOHOL</v>
@@ -13892,7 +13892,7 @@
         <v>24E-175</v>
       </c>
       <c r="B218" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C218" t="str">
         <v>VICTORIANO B. TIROL III AND WILL TYRON B. TIROL</v>
@@ -13954,7 +13954,7 @@
         <v>24E-176</v>
       </c>
       <c r="B219" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C219" t="str">
         <v>VICTORIANO B. TIROL III AND WILL TYRON B. TIROL</v>
@@ -14016,7 +14016,7 @@
         <v>97-1371</v>
       </c>
       <c r="B220" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C220" t="str">
         <v/>
@@ -14078,7 +14078,7 @@
         <v>VII-14-INQ-191-360</v>
       </c>
       <c r="B221" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C221" t="str">
         <v>PNP - TAGBILARAN CITY</v>
@@ -14140,7 +14140,7 @@
         <v>VII-14-INV-22B-037</v>
       </c>
       <c r="B222" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C222" t="str">
         <v>NICOLE OPENDO y GALES</v>
@@ -14202,7 +14202,7 @@
         <v>VII-14-INV-22B-038</v>
       </c>
       <c r="B223" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C223" t="str">
         <v>NICOLE OPENDO y GALES</v>
@@ -14264,7 +14264,7 @@
         <v>VII-14-INV-22B-039</v>
       </c>
       <c r="B224" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C224" t="str">
         <v>NICOLE OPENDO y GALES</v>
@@ -14326,7 +14326,7 @@
         <v>VII-14-INV-22B-040</v>
       </c>
       <c r="B225" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C225" t="str">
         <v>NICOLE OPENDO y GALES</v>
@@ -14388,7 +14388,7 @@
         <v>3636</v>
       </c>
       <c r="B226" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C226" t="str">
         <v/>
@@ -14450,7 +14450,7 @@
         <v>3341</v>
       </c>
       <c r="B227" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C227" t="str">
         <v/>
@@ -14512,7 +14512,7 @@
         <v>VII-14-INQ-22G-131</v>
       </c>
       <c r="B228" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C228" t="str">
         <v>PNP-TAGBILARAN CITY</v>
@@ -14636,7 +14636,7 @@
         <v>VII-14-INV-22L-453</v>
       </c>
       <c r="B230" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C230" t="str">
         <v>TAMPOS, MARIA IVY R.</v>
@@ -14822,7 +14822,7 @@
         <v>3430</v>
       </c>
       <c r="B233" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C233" t="str">
         <v/>
@@ -14884,7 +14884,7 @@
         <v>98-1063</v>
       </c>
       <c r="B234" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C234" t="str">
         <v/>
@@ -14946,7 +14946,7 @@
         <v>98-1063-A</v>
       </c>
       <c r="B235" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C235" t="str">
         <v/>
@@ -15008,7 +15008,7 @@
         <v>97-360</v>
       </c>
       <c r="B236" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C236" t="str">
         <v/>
@@ -15070,7 +15070,7 @@
         <v>97-361</v>
       </c>
       <c r="B237" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C237" t="str">
         <v/>
@@ -15132,7 +15132,7 @@
         <v>97-362</v>
       </c>
       <c r="B238" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C238" t="str">
         <v/>
@@ -15194,7 +15194,7 @@
         <v>3633</v>
       </c>
       <c r="B239" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C239" t="str">
         <v/>
@@ -15256,7 +15256,7 @@
         <v>362</v>
       </c>
       <c r="B240" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C240" t="str">
         <v/>
@@ -15380,7 +15380,7 @@
         <v>VII-14-INQ-19B-005</v>
       </c>
       <c r="B242" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C242" t="str">
         <v>NBI, TAGBILARAN CITY</v>
@@ -15442,7 +15442,7 @@
         <v>97-1337</v>
       </c>
       <c r="B243" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C243" t="str">
         <v/>
@@ -15566,7 +15566,7 @@
         <v>VII-14-INV-24I-286</v>
       </c>
       <c r="B245" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C245" t="str">
         <v>XU, FLORIE MUNEZ</v>
@@ -15628,7 +15628,7 @@
         <v>VII-14-INV-24I-287</v>
       </c>
       <c r="B246" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C246" t="str">
         <v>XU, FLORIE MUNEZ</v>
@@ -15690,7 +15690,7 @@
         <v>VII-14-INV-24I-288</v>
       </c>
       <c r="B247" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C247" t="str">
         <v>XU, FLORIE MUNEZ</v>
@@ -15938,7 +15938,7 @@
         <v>95-999</v>
       </c>
       <c r="B251" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C251" t="str">
         <v/>
@@ -16000,7 +16000,7 @@
         <v>24l-224</v>
       </c>
       <c r="B252" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C252" t="str">
         <v>LAIZA LOPEZ y BAUTISTA</v>
@@ -16062,7 +16062,7 @@
         <v>VII-14-INV-20J-284</v>
       </c>
       <c r="B253" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C253" t="str">
         <v>SSS-TAGBILARAN  CITY</v>
@@ -16124,7 +16124,7 @@
         <v>VII-14-INQ-19K-456</v>
       </c>
       <c r="B254" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C254" t="str">
         <v>BPPO, PIB, TAGBILARAN CITY</v>
@@ -16248,7 +16248,7 @@
         <v>VII-14-INV-22C-113</v>
       </c>
       <c r="B256" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C256" t="str">
         <v>ALBELDA, ANALOU S.</v>
@@ -16310,7 +16310,7 @@
         <v>VII-14-INQ-19L-476</v>
       </c>
       <c r="B257" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C257" t="str">
         <v>TAGB. CITY PNP</v>
@@ -16372,7 +16372,7 @@
         <v>VII-14-INQ-19L-336</v>
       </c>
       <c r="B258" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C258" t="str">
         <v>PNP, BOHOL</v>
@@ -16434,7 +16434,7 @@
         <v>VII-14-INQ-19I-336</v>
       </c>
       <c r="B259" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C259" t="str">
         <v>PNP, BOHOL</v>
@@ -16496,7 +16496,7 @@
         <v>VII-14-INQ-20K-409</v>
       </c>
       <c r="B260" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C260" t="str">
         <v>PNP TAGBILARAN CITY</v>
@@ -16558,7 +16558,7 @@
         <v>VII-14-INQ-20B-57</v>
       </c>
       <c r="B261" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C261" t="str">
         <v>PNP, BOHOL</v>
@@ -16620,7 +16620,7 @@
         <v>97-2372</v>
       </c>
       <c r="B262" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C262" t="str">
         <v/>
@@ -16682,7 +16682,7 @@
         <v>97-2373</v>
       </c>
       <c r="B263" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C263" t="str">
         <v/>
@@ -16744,7 +16744,7 @@
         <v>97-2374</v>
       </c>
       <c r="B264" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C264" t="str">
         <v/>
@@ -16868,7 +16868,7 @@
         <v>97-1622-A</v>
       </c>
       <c r="B266" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C266" t="str">
         <v/>
@@ -16930,7 +16930,7 @@
         <v>VII-14-INV-22H-328</v>
       </c>
       <c r="B267" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C267" t="str">
         <v>PDEA-BOHOL</v>
@@ -17054,7 +17054,7 @@
         <v>VII-14-INV-18K-252</v>
       </c>
       <c r="B269" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C269" t="str">
         <v>NBI, BOHOL                                            REP BY: RENNAN AUGUSTUS OLIVA</v>
@@ -17116,7 +17116,7 @@
         <v>VII-14-INV-18K-253</v>
       </c>
       <c r="B270" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C270" t="str">
         <v>NBI, BOHOL                                            REP BY: RENNAN AUGUSTUS OLIVA</v>
@@ -17240,7 +17240,7 @@
         <v>97-420</v>
       </c>
       <c r="B272" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C272" t="str">
         <v/>
@@ -17302,7 +17302,7 @@
         <v>97-421</v>
       </c>
       <c r="B273" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C273" t="str">
         <v/>
@@ -17364,7 +17364,7 @@
         <v>96-4164</v>
       </c>
       <c r="B274" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C274" t="str">
         <v/>
@@ -17426,7 +17426,7 @@
         <v>96-4165</v>
       </c>
       <c r="B275" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C275" t="str">
         <v/>
@@ -17488,7 +17488,7 @@
         <v>96-141</v>
       </c>
       <c r="B276" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C276" t="str">
         <v/>
@@ -17550,7 +17550,7 @@
         <v>96-1539</v>
       </c>
       <c r="B277" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C277" t="str">
         <v/>
@@ -17612,7 +17612,7 @@
         <v>96-1540</v>
       </c>
       <c r="B278" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C278" t="str">
         <v/>
@@ -17674,7 +17674,7 @@
         <v>96-1542</v>
       </c>
       <c r="B279" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C279" t="str">
         <v/>
@@ -17736,7 +17736,7 @@
         <v>96-1287</v>
       </c>
       <c r="B280" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C280" t="str">
         <v/>
@@ -17798,7 +17798,7 @@
         <v>96-1287-A</v>
       </c>
       <c r="B281" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C281" t="str">
         <v/>
@@ -18108,7 +18108,7 @@
         <v>VII-14-INV-22K-415</v>
       </c>
       <c r="B286" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C286" t="str">
         <v>BANAIS, PANFILO &amp; ANGALOT, CHRISTIAN</v>
@@ -18604,7 +18604,7 @@
         <v>VII-14-INQ-24E-103</v>
       </c>
       <c r="B294" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C294" t="str">
         <v>PNP-TABILARAN CITY</v>
@@ -18666,7 +18666,7 @@
         <v>VII-14-INQ-24E-104</v>
       </c>
       <c r="B295" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C295" t="str">
         <v>PNP-TABILARAN CITY</v>
@@ -18852,7 +18852,7 @@
         <v>VII-14-INQ-24K-311</v>
       </c>
       <c r="B298" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C298" t="str">
         <v>PNP-TABILARAN CITY</v>
@@ -18914,7 +18914,7 @@
         <v>VII-14-INQ-24K-312</v>
       </c>
       <c r="B299" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C299" t="str">
         <v>PNP-TABILARAN CITY</v>
@@ -18976,7 +18976,7 @@
         <v>VII-14-INQ-19I-351</v>
       </c>
       <c r="B300" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C300" t="str">
         <v>PNP-TABILARAN CITY</v>
@@ -19038,7 +19038,7 @@
         <v>VII-14-INQ-19I-350</v>
       </c>
       <c r="B301" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C301" t="str">
         <v>PNP-TABILARAN CITY</v>
@@ -19100,7 +19100,7 @@
         <v>VII-14-INQ-19D-164</v>
       </c>
       <c r="B302" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C302" t="str">
         <v>TAGBILARAN CITY POLICE</v>
@@ -19162,7 +19162,7 @@
         <v>VII-14-INV-17J-0328</v>
       </c>
       <c r="B303" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C303" t="str">
         <v/>
@@ -19224,7 +19224,7 @@
         <v>VII-14-INV-17J-0358</v>
       </c>
       <c r="B304" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C304" t="str">
         <v/>
@@ -19286,7 +19286,7 @@
         <v>VII-14-INV-17J-0357</v>
       </c>
       <c r="B305" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C305" t="str">
         <v/>
@@ -19348,7 +19348,7 @@
         <v>INV-14-INV-17J-0303</v>
       </c>
       <c r="B306" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C306" t="str">
         <v>MAMAC, PATRICK SISTER Y.</v>
@@ -19410,7 +19410,7 @@
         <v>VII-14-INV-24I-289</v>
       </c>
       <c r="B307" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C307" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19472,7 +19472,7 @@
         <v>VII-14-INV-24I-290</v>
       </c>
       <c r="B308" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C308" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19534,7 +19534,7 @@
         <v>VII-14-INV-24I-291</v>
       </c>
       <c r="B309" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C309" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19596,7 +19596,7 @@
         <v>VII-14-INV-24I-292</v>
       </c>
       <c r="B310" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C310" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19658,7 +19658,7 @@
         <v>VII-14-INV-24I-293</v>
       </c>
       <c r="B311" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C311" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19720,7 +19720,7 @@
         <v>VII-14-INV-24I-294</v>
       </c>
       <c r="B312" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C312" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19782,7 +19782,7 @@
         <v>VII-14-INV-24I-295</v>
       </c>
       <c r="B313" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C313" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19844,7 +19844,7 @@
         <v>VII-14-INV-24I-296</v>
       </c>
       <c r="B314" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C314" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19906,7 +19906,7 @@
         <v>VII-14-INV-24I-297</v>
       </c>
       <c r="B315" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C315" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19968,7 +19968,7 @@
         <v>VII-14-INV-24I-298</v>
       </c>
       <c r="B316" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C316" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -20030,7 +20030,7 @@
         <v>VII-14-INV-24I-299</v>
       </c>
       <c r="B317" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C317" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -20092,7 +20092,7 @@
         <v>VII-14-INV-24I-300</v>
       </c>
       <c r="B318" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C318" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -20154,7 +20154,7 @@
         <v>VII-14-INV-24I-301</v>
       </c>
       <c r="B319" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C319" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -20216,7 +20216,7 @@
         <v>VII-14-INQ-19F-201 C</v>
       </c>
       <c r="B320" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C320" t="str">
         <v>TAGBILARAN CITY POLICE STATION</v>
@@ -20340,7 +20340,7 @@
         <v>VII-14-INQ-24J-258</v>
       </c>
       <c r="B322" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C322" t="str">
         <v>PNP- TAGBILARAN CITY</v>
@@ -20402,7 +20402,7 @@
         <v>96-3001-3003</v>
       </c>
       <c r="B323" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C323" t="str">
         <v/>
@@ -20712,7 +20712,7 @@
         <v>97-251-253</v>
       </c>
       <c r="B328" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C328" t="str">
         <v/>
@@ -20774,7 +20774,7 @@
         <v>97-254-256</v>
       </c>
       <c r="B329" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C329" t="str">
         <v/>
@@ -20836,7 +20836,7 @@
         <v>VII-14-INQ-20J-406</v>
       </c>
       <c r="B330" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C330" t="str">
         <v>BUQUIL, JONIEL</v>
@@ -20898,7 +20898,7 @@
         <v>94-219</v>
       </c>
       <c r="B331" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C331" t="str">
         <v/>
@@ -21580,7 +21580,7 @@
         <v>96-4512-4514</v>
       </c>
       <c r="B342" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C342" t="str">
         <v/>
@@ -21704,7 +21704,7 @@
         <v>VII-14-INQ-22F-116</v>
       </c>
       <c r="B344" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C344" t="str">
         <v>BPPO, PIU BOHOL</v>
@@ -21766,7 +21766,7 @@
         <v>VII-14-INQ-22F-116</v>
       </c>
       <c r="B345" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C345" t="str">
         <v>BPPO, PIU BOHOL</v>
@@ -21828,7 +21828,7 @@
         <v>VII-14-INQ-22F-118</v>
       </c>
       <c r="B346" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C346" t="str">
         <v>BPPO, PIU BOHOL</v>
@@ -21890,7 +21890,7 @@
         <v>VII-14-INQ-22F-118</v>
       </c>
       <c r="B347" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C347" t="str">
         <v>BPPO, PIU BOHOL</v>
@@ -22262,7 +22262,7 @@
         <v>92-433</v>
       </c>
       <c r="B353" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C353" t="str">
         <v/>
@@ -22324,7 +22324,7 @@
         <v>96-1345</v>
       </c>
       <c r="B354" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C354" t="str">
         <v/>
@@ -22386,7 +22386,7 @@
         <v>99-290</v>
       </c>
       <c r="B355" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C355" t="str">
         <v/>
@@ -22510,7 +22510,7 @@
         <v>VII-14-INQ-18l-174</v>
       </c>
       <c r="B357" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C357" t="str">
         <v>PIB-SOG Bohol</v>
@@ -22572,7 +22572,7 @@
         <v>VII-14-INQ-18l-177</v>
       </c>
       <c r="B358" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C358" t="str">
         <v>PIB-SOG Bohol</v>
@@ -22758,7 +22758,7 @@
         <v>VII-14-INV-20J-275</v>
       </c>
       <c r="B361" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C361" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -22820,7 +22820,7 @@
         <v>VII-14-INV-20J-276</v>
       </c>
       <c r="B362" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C362" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -22882,7 +22882,7 @@
         <v>VII-14-INV-20J-277</v>
       </c>
       <c r="B363" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C363" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -22944,7 +22944,7 @@
         <v>VII-14-INV-20J-278</v>
       </c>
       <c r="B364" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C364" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -23006,7 +23006,7 @@
         <v>VII-14-INV-20J-279</v>
       </c>
       <c r="B365" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C365" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -23068,7 +23068,7 @@
         <v>VII-14-INV-20J-280</v>
       </c>
       <c r="B366" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C366" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -23130,7 +23130,7 @@
         <v>VII-14-INV-20J-281</v>
       </c>
       <c r="B367" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C367" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -23192,7 +23192,7 @@
         <v>VII-14-INV-20J-283</v>
       </c>
       <c r="B368" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C368" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -23254,7 +23254,7 @@
         <v>96-1607</v>
       </c>
       <c r="B369" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C369" t="str">
         <v/>
@@ -23316,7 +23316,7 @@
         <v>96-1607-A</v>
       </c>
       <c r="B370" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C370" t="str">
         <v/>
@@ -23378,7 +23378,7 @@
         <v>24J-240</v>
       </c>
       <c r="B371" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C371" t="str">
         <v>CITY PNP-TAGBILARAN CITY</v>
@@ -23440,7 +23440,7 @@
         <v>24J-241</v>
       </c>
       <c r="B372" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C372" t="str">
         <v>CITY PNP-TAGBILARAN CITY</v>
@@ -23626,7 +23626,7 @@
         <v>VII-14-INQ-21l-191</v>
       </c>
       <c r="B375" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C375" t="str">
         <v>PNP-TAGBILARAN CITY</v>
@@ -23688,7 +23688,7 @@
         <v>VII-14-INQ-21l-192</v>
       </c>
       <c r="B376" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C376" t="str">
         <v>PNP-TAGBILARAN CITY</v>
@@ -23750,7 +23750,7 @@
         <v>96-1820</v>
       </c>
       <c r="B377" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C377" t="str">
         <v/>
@@ -23812,7 +23812,7 @@
         <v>96-1821</v>
       </c>
       <c r="B378" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C378" t="str">
         <v/>
@@ -23874,7 +23874,7 @@
         <v>96-1822</v>
       </c>
       <c r="B379" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C379" t="str">
         <v/>
@@ -23936,7 +23936,7 @@
         <v>96-772</v>
       </c>
       <c r="B380" t="str">
-        <v>April 9, 2026</v>
+        <v>April 10, 2026</v>
       </c>
       <c r="C380" t="str">
         <v/>

</xml_diff>

<commit_message>
fixed the date filed of cases when uploading
</commit_message>
<xml_diff>
--- a/uploads/cases.xlsx
+++ b/uploads/cases.xlsx
@@ -500,7 +500,7 @@
         <v>VII-14-INQ-20I-361</v>
       </c>
       <c r="B2" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C2" t="str">
         <v>TAGBILARAN CITY PNP</v>
@@ -562,7 +562,7 @@
         <v>VII-14-INQ-20I-360</v>
       </c>
       <c r="B3" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C3" t="str">
         <v>TAGBILARAN CITY PNP</v>
@@ -934,7 +934,7 @@
         <v>2005-19</v>
       </c>
       <c r="B9" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C9" t="str">
         <v/>
@@ -996,7 +996,7 @@
         <v>2006-45</v>
       </c>
       <c r="B10" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C10" t="str">
         <v/>
@@ -1120,7 +1120,7 @@
         <v>VII-14-INQ-20A-04</v>
       </c>
       <c r="B12" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C12" t="str">
         <v>SALARDA, MYRA A.</v>
@@ -1306,7 +1306,7 @@
         <v>96-3427-3429</v>
       </c>
       <c r="B15" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C15" t="str">
         <v/>
@@ -1430,7 +1430,7 @@
         <v>3434</v>
       </c>
       <c r="B17" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C17" t="str">
         <v/>
@@ -2050,7 +2050,7 @@
         <v>VII-14-INV-22D-071</v>
       </c>
       <c r="B27" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C27" t="str">
         <v>CIDG-BOHOL</v>
@@ -2112,7 +2112,7 @@
         <v>VII-14-INV-22D-070</v>
       </c>
       <c r="B28" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C28" t="str">
         <v>CIDG-BOHOL</v>
@@ -2174,7 +2174,7 @@
         <v>VII-14-INQ-17A-027</v>
       </c>
       <c r="B29" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C29" t="str">
         <v/>
@@ -2360,7 +2360,7 @@
         <v>24H-260</v>
       </c>
       <c r="B32" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C32" t="str">
         <v>CADAYDAY, NEMESIA</v>
@@ -2422,7 +2422,7 @@
         <v>24H-260</v>
       </c>
       <c r="B33" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C33" t="str">
         <v>CADAYDAY,NEMESIA</v>
@@ -2484,7 +2484,7 @@
         <v>24H-261</v>
       </c>
       <c r="B34" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C34" t="str">
         <v>ALIVIADO, KHY</v>
@@ -2546,7 +2546,7 @@
         <v>24H-261</v>
       </c>
       <c r="B35" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C35" t="str">
         <v>CADAYDAY,NEMESIA</v>
@@ -2608,7 +2608,7 @@
         <v>96-228</v>
       </c>
       <c r="B36" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C36" t="str">
         <v/>
@@ -2670,7 +2670,7 @@
         <v>96-229</v>
       </c>
       <c r="B37" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C37" t="str">
         <v/>
@@ -2732,7 +2732,7 @@
         <v>96-230</v>
       </c>
       <c r="B38" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C38" t="str">
         <v/>
@@ -2794,7 +2794,7 @@
         <v>VII-14-INV-2OL-366</v>
       </c>
       <c r="B39" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C39" t="str">
         <v>PNP - TAGBILARAN CITY</v>
@@ -2980,7 +2980,7 @@
         <v>96-306</v>
       </c>
       <c r="B42" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C42" t="str">
         <v/>
@@ -3042,7 +3042,7 @@
         <v>96-307</v>
       </c>
       <c r="B43" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C43" t="str">
         <v/>
@@ -3104,7 +3104,7 @@
         <v>96-308</v>
       </c>
       <c r="B44" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C44" t="str">
         <v/>
@@ -3352,7 +3352,7 @@
         <v>VII-14-INQ-221-197</v>
       </c>
       <c r="B48" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C48" t="str">
         <v>PDEA-BOHOL</v>
@@ -3476,7 +3476,7 @@
         <v>VII-14-INQ-221-196</v>
       </c>
       <c r="B50" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C50" t="str">
         <v>PDEA-BOHOL</v>
@@ -3538,7 +3538,7 @@
         <v>3145</v>
       </c>
       <c r="B51" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C51" t="str">
         <v/>
@@ -3600,7 +3600,7 @@
         <v>3144</v>
       </c>
       <c r="B52" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C52" t="str">
         <v/>
@@ -3786,7 +3786,7 @@
         <v>VII-14-INV-175-0325</v>
       </c>
       <c r="B55" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C55" t="str">
         <v/>
@@ -3972,7 +3972,7 @@
         <v>VII-14-INV-20A-27</v>
       </c>
       <c r="B58" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C58" t="str">
         <v>CIDG-BOHOL</v>
@@ -4034,7 +4034,7 @@
         <v>VII-14-INV-20A-26</v>
       </c>
       <c r="B59" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C59" t="str">
         <v>CIDG-BOHOL</v>
@@ -4158,7 +4158,7 @@
         <v>2000-129</v>
       </c>
       <c r="B61" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C61" t="str">
         <v/>
@@ -4220,7 +4220,7 @@
         <v>2000-130</v>
       </c>
       <c r="B62" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C62" t="str">
         <v/>
@@ -4282,7 +4282,7 @@
         <v>2000-131</v>
       </c>
       <c r="B63" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C63" t="str">
         <v/>
@@ -4344,7 +4344,7 @@
         <v>2000-132</v>
       </c>
       <c r="B64" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C64" t="str">
         <v/>
@@ -4406,7 +4406,7 @@
         <v>2000-133</v>
       </c>
       <c r="B65" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C65" t="str">
         <v/>
@@ -4468,7 +4468,7 @@
         <v>2000-134</v>
       </c>
       <c r="B66" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C66" t="str">
         <v/>
@@ -4530,7 +4530,7 @@
         <v>2000-135</v>
       </c>
       <c r="B67" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C67" t="str">
         <v/>
@@ -4592,7 +4592,7 @@
         <v>2000-136</v>
       </c>
       <c r="B68" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C68" t="str">
         <v/>
@@ -4654,7 +4654,7 @@
         <v>2000-137</v>
       </c>
       <c r="B69" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C69" t="str">
         <v/>
@@ -4716,7 +4716,7 @@
         <v>2000-138</v>
       </c>
       <c r="B70" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C70" t="str">
         <v/>
@@ -4778,7 +4778,7 @@
         <v>2000-139</v>
       </c>
       <c r="B71" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C71" t="str">
         <v/>
@@ -4840,7 +4840,7 @@
         <v>VII-14-INQ-24K-285</v>
       </c>
       <c r="B72" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C72" t="str">
         <v>NBI-CEBU OFFICE -MANDAUE CITY</v>
@@ -4902,7 +4902,7 @@
         <v>99-317</v>
       </c>
       <c r="B73" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C73" t="str">
         <v/>
@@ -4964,7 +4964,7 @@
         <v>VII-14-INV-20H-207</v>
       </c>
       <c r="B74" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C74" t="str">
         <v>BINAMIRA, GARRY NOEL E.</v>
@@ -5026,7 +5026,7 @@
         <v>24J-242</v>
       </c>
       <c r="B75" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C75" t="str">
         <v>PDEA-BOHOL</v>
@@ -5088,7 +5088,7 @@
         <v>24J-243</v>
       </c>
       <c r="B76" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C76" t="str">
         <v>PDEA-BOHOL</v>
@@ -5150,7 +5150,7 @@
         <v>24J-244</v>
       </c>
       <c r="B77" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C77" t="str">
         <v>PDEA-BOHOL</v>
@@ -5212,7 +5212,7 @@
         <v>24J-245</v>
       </c>
       <c r="B78" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C78" t="str">
         <v>PDEA-BOHOL</v>
@@ -5336,7 +5336,7 @@
         <v>89-289 89-289-A 89-289-B 89-289-C 89-289-D</v>
       </c>
       <c r="B80" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C80" t="str">
         <v/>
@@ -5398,7 +5398,7 @@
         <v>VII-14-INV-21A-079</v>
       </c>
       <c r="B81" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C81" t="str">
         <v>STARLITE MARINE INDUSTRIAL SERVICES CORP.</v>
@@ -5460,7 +5460,7 @@
         <v>24K-300</v>
       </c>
       <c r="B82" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C82" t="str">
         <v>PNP - TAGBILARAN CITY</v>
@@ -6452,7 +6452,7 @@
         <v>96-1464</v>
       </c>
       <c r="B98" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C98" t="str">
         <v/>
@@ -6700,7 +6700,7 @@
         <v>92-195</v>
       </c>
       <c r="B102" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C102" t="str">
         <v/>
@@ -6762,7 +6762,7 @@
         <v>VII-14-INV-24B-55</v>
       </c>
       <c r="B103" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C103" t="str">
         <v>BAJA, NOEL B.</v>
@@ -6824,7 +6824,7 @@
         <v>86-226</v>
       </c>
       <c r="B104" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C104" t="str">
         <v/>
@@ -6886,7 +6886,7 @@
         <v>97-3828</v>
       </c>
       <c r="B105" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C105" t="str">
         <v/>
@@ -6948,7 +6948,7 @@
         <v>97-3829</v>
       </c>
       <c r="B106" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C106" t="str">
         <v/>
@@ -7010,7 +7010,7 @@
         <v>97-3830</v>
       </c>
       <c r="B107" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C107" t="str">
         <v/>
@@ -7072,7 +7072,7 @@
         <v>97-3831</v>
       </c>
       <c r="B108" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C108" t="str">
         <v/>
@@ -7754,7 +7754,7 @@
         <v>3510</v>
       </c>
       <c r="B119" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C119" t="str">
         <v/>
@@ -7816,7 +7816,7 @@
         <v>96-2673</v>
       </c>
       <c r="B120" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C120" t="str">
         <v/>
@@ -7878,7 +7878,7 @@
         <v>96-2674</v>
       </c>
       <c r="B121" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C121" t="str">
         <v/>
@@ -7940,7 +7940,7 @@
         <v>96-2675</v>
       </c>
       <c r="B122" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C122" t="str">
         <v/>
@@ -8002,7 +8002,7 @@
         <v>97-3037</v>
       </c>
       <c r="B123" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C123" t="str">
         <v/>
@@ -8064,7 +8064,7 @@
         <v>97-3038</v>
       </c>
       <c r="B124" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C124" t="str">
         <v/>
@@ -8126,7 +8126,7 @@
         <v>97-3039</v>
       </c>
       <c r="B125" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C125" t="str">
         <v/>
@@ -8188,7 +8188,7 @@
         <v>97-1336</v>
       </c>
       <c r="B126" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C126" t="str">
         <v/>
@@ -8250,7 +8250,7 @@
         <v>97-1336</v>
       </c>
       <c r="B127" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C127" t="str">
         <v/>
@@ -8374,7 +8374,7 @@
         <v>97-1339</v>
       </c>
       <c r="B129" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C129" t="str">
         <v/>
@@ -8436,7 +8436,7 @@
         <v>97-1340</v>
       </c>
       <c r="B130" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C130" t="str">
         <v/>
@@ -8498,7 +8498,7 @@
         <v>97-1341</v>
       </c>
       <c r="B131" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C131" t="str">
         <v/>
@@ -8560,7 +8560,7 @@
         <v>96-2554</v>
       </c>
       <c r="B132" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C132" t="str">
         <v/>
@@ -8622,7 +8622,7 @@
         <v>96-2555</v>
       </c>
       <c r="B133" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C133" t="str">
         <v/>
@@ -8684,7 +8684,7 @@
         <v>96-2556</v>
       </c>
       <c r="B134" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C134" t="str">
         <v/>
@@ -8746,7 +8746,7 @@
         <v>96-2557</v>
       </c>
       <c r="B135" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C135" t="str">
         <v/>
@@ -8808,7 +8808,7 @@
         <v>96-2558</v>
       </c>
       <c r="B136" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C136" t="str">
         <v/>
@@ -8870,7 +8870,7 @@
         <v>24l-222</v>
       </c>
       <c r="B137" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C137" t="str">
         <v>TAGBILARAN CITY - PNP</v>
@@ -8932,7 +8932,7 @@
         <v>24l-223</v>
       </c>
       <c r="B138" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C138" t="str">
         <v>TAGBILARAN CITY - PNP</v>
@@ -9366,7 +9366,7 @@
         <v>97-397</v>
       </c>
       <c r="B145" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C145" t="str">
         <v/>
@@ -9428,7 +9428,7 @@
         <v>2005-537</v>
       </c>
       <c r="B146" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C146" t="str">
         <v/>
@@ -9738,7 +9738,7 @@
         <v>2002-999</v>
       </c>
       <c r="B151" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C151" t="str">
         <v/>
@@ -9800,7 +9800,7 @@
         <v>2002-1000</v>
       </c>
       <c r="B152" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C152" t="str">
         <v/>
@@ -9862,7 +9862,7 @@
         <v>2002-1001</v>
       </c>
       <c r="B153" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C153" t="str">
         <v/>
@@ -9924,7 +9924,7 @@
         <v>2002-1002</v>
       </c>
       <c r="B154" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C154" t="str">
         <v/>
@@ -9986,7 +9986,7 @@
         <v>3961</v>
       </c>
       <c r="B155" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C155" t="str">
         <v/>
@@ -10048,7 +10048,7 @@
         <v>VII-14-INQ-23B-061</v>
       </c>
       <c r="B156" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C156" t="str">
         <v>PIU-BOHOL PPO</v>
@@ -10110,7 +10110,7 @@
         <v>VII-14-INQ-23B-061</v>
       </c>
       <c r="B157" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C157" t="str">
         <v>PIU BOHOL PPO</v>
@@ -10172,7 +10172,7 @@
         <v>VII-14-INQ-23B-062</v>
       </c>
       <c r="B158" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C158" t="str">
         <v>PIU-BOHOL PPO</v>
@@ -10234,7 +10234,7 @@
         <v>VII-14-INQ-23B-062</v>
       </c>
       <c r="B159" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C159" t="str">
         <v>PIU BOHOL PPO</v>
@@ -10420,7 +10420,7 @@
         <v>93-463</v>
       </c>
       <c r="B162" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C162" t="str">
         <v/>
@@ -10482,7 +10482,7 @@
         <v>93-464</v>
       </c>
       <c r="B163" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C163" t="str">
         <v/>
@@ -10544,7 +10544,7 @@
         <v>96-1680</v>
       </c>
       <c r="B164" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C164" t="str">
         <v/>
@@ -10606,7 +10606,7 @@
         <v>96-1681</v>
       </c>
       <c r="B165" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C165" t="str">
         <v/>
@@ -10668,7 +10668,7 @@
         <v>96-1682</v>
       </c>
       <c r="B166" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C166" t="str">
         <v/>
@@ -10730,7 +10730,7 @@
         <v>96-1697</v>
       </c>
       <c r="B167" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C167" t="str">
         <v/>
@@ -10792,7 +10792,7 @@
         <v>96-1698</v>
       </c>
       <c r="B168" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C168" t="str">
         <v/>
@@ -10854,7 +10854,7 @@
         <v>96-1699</v>
       </c>
       <c r="B169" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C169" t="str">
         <v/>
@@ -10978,7 +10978,7 @@
         <v>VII-14-INQ-24J-257</v>
       </c>
       <c r="B171" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C171" t="str">
         <v>PNP-TAGBILARAN CITY</v>
@@ -11040,7 +11040,7 @@
         <v>VII-14-INQ-24J-257</v>
       </c>
       <c r="B172" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C172" t="str">
         <v>PNP- TAGBILARAN CITY</v>
@@ -11102,7 +11102,7 @@
         <v>96-831</v>
       </c>
       <c r="B173" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C173" t="str">
         <v/>
@@ -11164,7 +11164,7 @@
         <v>VII-14-INV-24J-316</v>
       </c>
       <c r="B174" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C174" t="str">
         <v>ROSALEJOS, ALFONSO LIGO</v>
@@ -11226,7 +11226,7 @@
         <v>VII-14-INV-24J-316 b</v>
       </c>
       <c r="B175" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C175" t="str">
         <v>ROSALEJOS, ALFONSO LIGO</v>
@@ -11288,7 +11288,7 @@
         <v>97-3034</v>
       </c>
       <c r="B176" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C176" t="str">
         <v/>
@@ -11350,7 +11350,7 @@
         <v>97-3035</v>
       </c>
       <c r="B177" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C177" t="str">
         <v/>
@@ -11412,7 +11412,7 @@
         <v>97-3036</v>
       </c>
       <c r="B178" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C178" t="str">
         <v/>
@@ -11474,7 +11474,7 @@
         <v>96-1724</v>
       </c>
       <c r="B179" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C179" t="str">
         <v/>
@@ -11536,7 +11536,7 @@
         <v>96-1725</v>
       </c>
       <c r="B180" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C180" t="str">
         <v/>
@@ -11598,7 +11598,7 @@
         <v>96-1726</v>
       </c>
       <c r="B181" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C181" t="str">
         <v/>
@@ -11660,7 +11660,7 @@
         <v>96-1574</v>
       </c>
       <c r="B182" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C182" t="str">
         <v/>
@@ -11722,7 +11722,7 @@
         <v>96-1575</v>
       </c>
       <c r="B183" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C183" t="str">
         <v/>
@@ -11784,7 +11784,7 @@
         <v>96-1576</v>
       </c>
       <c r="B184" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C184" t="str">
         <v/>
@@ -11846,7 +11846,7 @@
         <v>98-004</v>
       </c>
       <c r="B185" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C185" t="str">
         <v/>
@@ -11908,7 +11908,7 @@
         <v>98-005</v>
       </c>
       <c r="B186" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C186" t="str">
         <v/>
@@ -12280,7 +12280,7 @@
         <v>VII-14-INQ-20K-408</v>
       </c>
       <c r="B192" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C192" t="str">
         <v>PNP-TAGBILARAN CITY</v>
@@ -12342,7 +12342,7 @@
         <v>VII-14-INQ-20K-408</v>
       </c>
       <c r="B193" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C193" t="str">
         <v>PNP TAGBILARAN CITY</v>
@@ -12466,7 +12466,7 @@
         <v>VII-14-INQ-19E-197</v>
       </c>
       <c r="B195" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C195" t="str">
         <v>TAGBILARAN CITY POLICE</v>
@@ -13396,7 +13396,7 @@
         <v>VII-14-INV-20E-99</v>
       </c>
       <c r="B210" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C210" t="str">
         <v>FERNANDEZ, EULALIA A.</v>
@@ -13458,7 +13458,7 @@
         <v>VII-14-INV-18D-0132</v>
       </c>
       <c r="B211" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C211" t="str">
         <v>FCB, REP BY: GALAB, ANTHONY B.</v>
@@ -13520,7 +13520,7 @@
         <v>VII-14-INV-17H-0230</v>
       </c>
       <c r="B212" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C212" t="str">
         <v>A-1-BY TAGASLING, JOSEPHINE B.</v>
@@ -13582,7 +13582,7 @@
         <v>VII-14-INV-17H-0230 -A</v>
       </c>
       <c r="B213" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C213" t="str">
         <v>A-1-BY TAGASLING, JOSEPHINE B.</v>
@@ -13644,7 +13644,7 @@
         <v>VII-14-INV-18K-445</v>
       </c>
       <c r="B214" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C214" t="str">
         <v>GALLA, JOHN S.</v>
@@ -13706,7 +13706,7 @@
         <v>VII-14-INV-20E-100</v>
       </c>
       <c r="B215" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C215" t="str">
         <v>FERNANDEZ, EULALIA A.</v>
@@ -13768,7 +13768,7 @@
         <v>VII-14-INV-21B-30</v>
       </c>
       <c r="B216" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C216" t="str">
         <v>CIDG-BOHOL</v>
@@ -13830,7 +13830,7 @@
         <v>VII-14-INV-21B-31</v>
       </c>
       <c r="B217" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C217" t="str">
         <v>CIDG-BOHOL</v>
@@ -13892,7 +13892,7 @@
         <v>24E-175</v>
       </c>
       <c r="B218" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C218" t="str">
         <v>VICTORIANO B. TIROL III AND WILL TYRON B. TIROL</v>
@@ -13954,7 +13954,7 @@
         <v>24E-176</v>
       </c>
       <c r="B219" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C219" t="str">
         <v>VICTORIANO B. TIROL III AND WILL TYRON B. TIROL</v>
@@ -14016,7 +14016,7 @@
         <v>97-1371</v>
       </c>
       <c r="B220" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C220" t="str">
         <v/>
@@ -14078,7 +14078,7 @@
         <v>VII-14-INQ-191-360</v>
       </c>
       <c r="B221" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C221" t="str">
         <v>PNP - TAGBILARAN CITY</v>
@@ -14140,7 +14140,7 @@
         <v>VII-14-INV-22B-037</v>
       </c>
       <c r="B222" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C222" t="str">
         <v>NICOLE OPENDO y GALES</v>
@@ -14202,7 +14202,7 @@
         <v>VII-14-INV-22B-038</v>
       </c>
       <c r="B223" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C223" t="str">
         <v>NICOLE OPENDO y GALES</v>
@@ -14264,7 +14264,7 @@
         <v>VII-14-INV-22B-039</v>
       </c>
       <c r="B224" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C224" t="str">
         <v>NICOLE OPENDO y GALES</v>
@@ -14326,7 +14326,7 @@
         <v>VII-14-INV-22B-040</v>
       </c>
       <c r="B225" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C225" t="str">
         <v>NICOLE OPENDO y GALES</v>
@@ -14388,7 +14388,7 @@
         <v>3636</v>
       </c>
       <c r="B226" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C226" t="str">
         <v/>
@@ -14450,7 +14450,7 @@
         <v>3341</v>
       </c>
       <c r="B227" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C227" t="str">
         <v/>
@@ -14512,7 +14512,7 @@
         <v>VII-14-INQ-22G-131</v>
       </c>
       <c r="B228" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C228" t="str">
         <v>PNP-TAGBILARAN CITY</v>
@@ -14636,7 +14636,7 @@
         <v>VII-14-INV-22L-453</v>
       </c>
       <c r="B230" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C230" t="str">
         <v>TAMPOS, MARIA IVY R.</v>
@@ -14822,7 +14822,7 @@
         <v>3430</v>
       </c>
       <c r="B233" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C233" t="str">
         <v/>
@@ -14884,7 +14884,7 @@
         <v>98-1063</v>
       </c>
       <c r="B234" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C234" t="str">
         <v/>
@@ -14946,7 +14946,7 @@
         <v>98-1063-A</v>
       </c>
       <c r="B235" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C235" t="str">
         <v/>
@@ -15008,7 +15008,7 @@
         <v>97-360</v>
       </c>
       <c r="B236" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C236" t="str">
         <v/>
@@ -15070,7 +15070,7 @@
         <v>97-361</v>
       </c>
       <c r="B237" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C237" t="str">
         <v/>
@@ -15132,7 +15132,7 @@
         <v>97-362</v>
       </c>
       <c r="B238" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C238" t="str">
         <v/>
@@ -15194,7 +15194,7 @@
         <v>3633</v>
       </c>
       <c r="B239" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C239" t="str">
         <v/>
@@ -15256,7 +15256,7 @@
         <v>362</v>
       </c>
       <c r="B240" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C240" t="str">
         <v/>
@@ -15380,7 +15380,7 @@
         <v>VII-14-INQ-19B-005</v>
       </c>
       <c r="B242" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C242" t="str">
         <v>NBI, TAGBILARAN CITY</v>
@@ -15442,7 +15442,7 @@
         <v>97-1337</v>
       </c>
       <c r="B243" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C243" t="str">
         <v/>
@@ -15566,7 +15566,7 @@
         <v>VII-14-INV-24I-286</v>
       </c>
       <c r="B245" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C245" t="str">
         <v>XU, FLORIE MUNEZ</v>
@@ -15628,7 +15628,7 @@
         <v>VII-14-INV-24I-287</v>
       </c>
       <c r="B246" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C246" t="str">
         <v>XU, FLORIE MUNEZ</v>
@@ -15690,7 +15690,7 @@
         <v>VII-14-INV-24I-288</v>
       </c>
       <c r="B247" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C247" t="str">
         <v>XU, FLORIE MUNEZ</v>
@@ -15814,7 +15814,7 @@
         <v>VII-14-INV 24B-45</v>
       </c>
       <c r="B249" t="str">
-        <v>February 13, 2024</v>
+        <v/>
       </c>
       <c r="C249" t="str">
         <v>TARIAO, ROSALINDA R.</v>
@@ -15876,7 +15876,7 @@
         <v>VII-14-INV 24B-45</v>
       </c>
       <c r="B250" t="str">
-        <v>February 13, 2024</v>
+        <v/>
       </c>
       <c r="C250" t="str">
         <v>TARIAO, ROSALINDA R.</v>
@@ -15938,7 +15938,7 @@
         <v>95-999</v>
       </c>
       <c r="B251" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C251" t="str">
         <v/>
@@ -16000,7 +16000,7 @@
         <v>24l-224</v>
       </c>
       <c r="B252" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C252" t="str">
         <v>LAIZA LOPEZ y BAUTISTA</v>
@@ -16062,7 +16062,7 @@
         <v>VII-14-INV-20J-284</v>
       </c>
       <c r="B253" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C253" t="str">
         <v>SSS-TAGBILARAN  CITY</v>
@@ -16124,7 +16124,7 @@
         <v>VII-14-INQ-19K-456</v>
       </c>
       <c r="B254" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C254" t="str">
         <v>BPPO, PIB, TAGBILARAN CITY</v>
@@ -16248,7 +16248,7 @@
         <v>VII-14-INV-22C-113</v>
       </c>
       <c r="B256" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C256" t="str">
         <v>ALBELDA, ANALOU S.</v>
@@ -16310,7 +16310,7 @@
         <v>VII-14-INQ-19L-476</v>
       </c>
       <c r="B257" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C257" t="str">
         <v>TAGB. CITY PNP</v>
@@ -16372,7 +16372,7 @@
         <v>VII-14-INQ-19L-336</v>
       </c>
       <c r="B258" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C258" t="str">
         <v>PNP, BOHOL</v>
@@ -16434,7 +16434,7 @@
         <v>VII-14-INQ-19I-336</v>
       </c>
       <c r="B259" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C259" t="str">
         <v>PNP, BOHOL</v>
@@ -16496,7 +16496,7 @@
         <v>VII-14-INQ-20K-409</v>
       </c>
       <c r="B260" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C260" t="str">
         <v>PNP TAGBILARAN CITY</v>
@@ -16558,7 +16558,7 @@
         <v>VII-14-INQ-20B-57</v>
       </c>
       <c r="B261" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C261" t="str">
         <v>PNP, BOHOL</v>
@@ -16620,7 +16620,7 @@
         <v>97-2372</v>
       </c>
       <c r="B262" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C262" t="str">
         <v/>
@@ -16682,7 +16682,7 @@
         <v>97-2373</v>
       </c>
       <c r="B263" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C263" t="str">
         <v/>
@@ -16744,7 +16744,7 @@
         <v>97-2374</v>
       </c>
       <c r="B264" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C264" t="str">
         <v/>
@@ -16868,7 +16868,7 @@
         <v>97-1622-A</v>
       </c>
       <c r="B266" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C266" t="str">
         <v/>
@@ -16930,7 +16930,7 @@
         <v>VII-14-INV-22H-328</v>
       </c>
       <c r="B267" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C267" t="str">
         <v>PDEA-BOHOL</v>
@@ -17054,7 +17054,7 @@
         <v>VII-14-INV-18K-252</v>
       </c>
       <c r="B269" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C269" t="str">
         <v>NBI, BOHOL                                            REP BY: RENNAN AUGUSTUS OLIVA</v>
@@ -17116,7 +17116,7 @@
         <v>VII-14-INV-18K-253</v>
       </c>
       <c r="B270" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C270" t="str">
         <v>NBI, BOHOL                                            REP BY: RENNAN AUGUSTUS OLIVA</v>
@@ -17240,7 +17240,7 @@
         <v>97-420</v>
       </c>
       <c r="B272" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C272" t="str">
         <v/>
@@ -17302,7 +17302,7 @@
         <v>97-421</v>
       </c>
       <c r="B273" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C273" t="str">
         <v/>
@@ -17364,7 +17364,7 @@
         <v>96-4164</v>
       </c>
       <c r="B274" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C274" t="str">
         <v/>
@@ -17426,7 +17426,7 @@
         <v>96-4165</v>
       </c>
       <c r="B275" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C275" t="str">
         <v/>
@@ -17488,7 +17488,7 @@
         <v>96-141</v>
       </c>
       <c r="B276" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C276" t="str">
         <v/>
@@ -17550,7 +17550,7 @@
         <v>96-1539</v>
       </c>
       <c r="B277" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C277" t="str">
         <v/>
@@ -17612,7 +17612,7 @@
         <v>96-1540</v>
       </c>
       <c r="B278" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C278" t="str">
         <v/>
@@ -17674,7 +17674,7 @@
         <v>96-1542</v>
       </c>
       <c r="B279" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C279" t="str">
         <v/>
@@ -17736,7 +17736,7 @@
         <v>96-1287</v>
       </c>
       <c r="B280" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C280" t="str">
         <v/>
@@ -17798,7 +17798,7 @@
         <v>96-1287-A</v>
       </c>
       <c r="B281" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C281" t="str">
         <v/>
@@ -18108,7 +18108,7 @@
         <v>VII-14-INV-22K-415</v>
       </c>
       <c r="B286" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C286" t="str">
         <v>BANAIS, PANFILO &amp; ANGALOT, CHRISTIAN</v>
@@ -18604,7 +18604,7 @@
         <v>VII-14-INQ-24E-103</v>
       </c>
       <c r="B294" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C294" t="str">
         <v>PNP-TABILARAN CITY</v>
@@ -18666,7 +18666,7 @@
         <v>VII-14-INQ-24E-104</v>
       </c>
       <c r="B295" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C295" t="str">
         <v>PNP-TABILARAN CITY</v>
@@ -18852,7 +18852,7 @@
         <v>VII-14-INQ-24K-311</v>
       </c>
       <c r="B298" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C298" t="str">
         <v>PNP-TABILARAN CITY</v>
@@ -18914,7 +18914,7 @@
         <v>VII-14-INQ-24K-312</v>
       </c>
       <c r="B299" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C299" t="str">
         <v>PNP-TABILARAN CITY</v>
@@ -18976,7 +18976,7 @@
         <v>VII-14-INQ-19I-351</v>
       </c>
       <c r="B300" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C300" t="str">
         <v>PNP-TABILARAN CITY</v>
@@ -19038,7 +19038,7 @@
         <v>VII-14-INQ-19I-350</v>
       </c>
       <c r="B301" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C301" t="str">
         <v>PNP-TABILARAN CITY</v>
@@ -19100,7 +19100,7 @@
         <v>VII-14-INQ-19D-164</v>
       </c>
       <c r="B302" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C302" t="str">
         <v>TAGBILARAN CITY POLICE</v>
@@ -19162,7 +19162,7 @@
         <v>VII-14-INV-17J-0328</v>
       </c>
       <c r="B303" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C303" t="str">
         <v/>
@@ -19224,7 +19224,7 @@
         <v>VII-14-INV-17J-0358</v>
       </c>
       <c r="B304" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C304" t="str">
         <v/>
@@ -19286,7 +19286,7 @@
         <v>VII-14-INV-17J-0357</v>
       </c>
       <c r="B305" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C305" t="str">
         <v/>
@@ -19348,7 +19348,7 @@
         <v>INV-14-INV-17J-0303</v>
       </c>
       <c r="B306" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C306" t="str">
         <v>MAMAC, PATRICK SISTER Y.</v>
@@ -19410,7 +19410,7 @@
         <v>VII-14-INV-24I-289</v>
       </c>
       <c r="B307" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C307" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19472,7 +19472,7 @@
         <v>VII-14-INV-24I-290</v>
       </c>
       <c r="B308" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C308" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19534,7 +19534,7 @@
         <v>VII-14-INV-24I-291</v>
       </c>
       <c r="B309" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C309" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19596,7 +19596,7 @@
         <v>VII-14-INV-24I-292</v>
       </c>
       <c r="B310" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C310" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19658,7 +19658,7 @@
         <v>VII-14-INV-24I-293</v>
       </c>
       <c r="B311" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C311" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19720,7 +19720,7 @@
         <v>VII-14-INV-24I-294</v>
       </c>
       <c r="B312" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C312" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19782,7 +19782,7 @@
         <v>VII-14-INV-24I-295</v>
       </c>
       <c r="B313" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C313" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19844,7 +19844,7 @@
         <v>VII-14-INV-24I-296</v>
       </c>
       <c r="B314" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C314" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19906,7 +19906,7 @@
         <v>VII-14-INV-24I-297</v>
       </c>
       <c r="B315" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C315" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -19968,7 +19968,7 @@
         <v>VII-14-INV-24I-298</v>
       </c>
       <c r="B316" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C316" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -20030,7 +20030,7 @@
         <v>VII-14-INV-24I-299</v>
       </c>
       <c r="B317" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C317" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -20092,7 +20092,7 @@
         <v>VII-14-INV-24I-300</v>
       </c>
       <c r="B318" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C318" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -20154,7 +20154,7 @@
         <v>VII-14-INV-24I-301</v>
       </c>
       <c r="B319" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C319" t="str">
         <v>VERGABERA, NORBERTO JR.</v>
@@ -20216,7 +20216,7 @@
         <v>VII-14-INQ-19F-201 C</v>
       </c>
       <c r="B320" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C320" t="str">
         <v>TAGBILARAN CITY POLICE STATION</v>
@@ -20340,7 +20340,7 @@
         <v>VII-14-INQ-24J-258</v>
       </c>
       <c r="B322" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C322" t="str">
         <v>PNP- TAGBILARAN CITY</v>
@@ -20402,7 +20402,7 @@
         <v>96-3001-3003</v>
       </c>
       <c r="B323" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C323" t="str">
         <v/>
@@ -20712,7 +20712,7 @@
         <v>97-251-253</v>
       </c>
       <c r="B328" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C328" t="str">
         <v/>
@@ -20774,7 +20774,7 @@
         <v>97-254-256</v>
       </c>
       <c r="B329" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C329" t="str">
         <v/>
@@ -20836,7 +20836,7 @@
         <v>VII-14-INQ-20J-406</v>
       </c>
       <c r="B330" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C330" t="str">
         <v>BUQUIL, JONIEL</v>
@@ -20898,7 +20898,7 @@
         <v>94-219</v>
       </c>
       <c r="B331" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C331" t="str">
         <v/>
@@ -21580,7 +21580,7 @@
         <v>96-4512-4514</v>
       </c>
       <c r="B342" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C342" t="str">
         <v/>
@@ -21704,7 +21704,7 @@
         <v>VII-14-INQ-22F-116</v>
       </c>
       <c r="B344" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C344" t="str">
         <v>BPPO, PIU BOHOL</v>
@@ -21766,7 +21766,7 @@
         <v>VII-14-INQ-22F-116</v>
       </c>
       <c r="B345" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C345" t="str">
         <v>BPPO, PIU BOHOL</v>
@@ -21828,7 +21828,7 @@
         <v>VII-14-INQ-22F-118</v>
       </c>
       <c r="B346" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C346" t="str">
         <v>BPPO, PIU BOHOL</v>
@@ -21890,7 +21890,7 @@
         <v>VII-14-INQ-22F-118</v>
       </c>
       <c r="B347" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C347" t="str">
         <v>BPPO, PIU BOHOL</v>
@@ -22262,7 +22262,7 @@
         <v>92-433</v>
       </c>
       <c r="B353" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C353" t="str">
         <v/>
@@ -22324,7 +22324,7 @@
         <v>96-1345</v>
       </c>
       <c r="B354" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C354" t="str">
         <v/>
@@ -22386,7 +22386,7 @@
         <v>99-290</v>
       </c>
       <c r="B355" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C355" t="str">
         <v/>
@@ -22510,7 +22510,7 @@
         <v>VII-14-INQ-18l-174</v>
       </c>
       <c r="B357" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C357" t="str">
         <v>PIB-SOG Bohol</v>
@@ -22572,7 +22572,7 @@
         <v>VII-14-INQ-18l-177</v>
       </c>
       <c r="B358" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C358" t="str">
         <v>PIB-SOG Bohol</v>
@@ -22758,7 +22758,7 @@
         <v>VII-14-INV-20J-275</v>
       </c>
       <c r="B361" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C361" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -22820,7 +22820,7 @@
         <v>VII-14-INV-20J-276</v>
       </c>
       <c r="B362" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C362" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -22882,7 +22882,7 @@
         <v>VII-14-INV-20J-277</v>
       </c>
       <c r="B363" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C363" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -22944,7 +22944,7 @@
         <v>VII-14-INV-20J-278</v>
       </c>
       <c r="B364" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C364" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -23006,7 +23006,7 @@
         <v>VII-14-INV-20J-279</v>
       </c>
       <c r="B365" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C365" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -23068,7 +23068,7 @@
         <v>VII-14-INV-20J-280</v>
       </c>
       <c r="B366" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C366" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -23130,7 +23130,7 @@
         <v>VII-14-INV-20J-281</v>
       </c>
       <c r="B367" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C367" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -23192,7 +23192,7 @@
         <v>VII-14-INV-20J-283</v>
       </c>
       <c r="B368" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C368" t="str">
         <v>PATTI MAE REGINE L. CLERIGO</v>
@@ -23254,7 +23254,7 @@
         <v>96-1607</v>
       </c>
       <c r="B369" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C369" t="str">
         <v/>
@@ -23316,7 +23316,7 @@
         <v>96-1607-A</v>
       </c>
       <c r="B370" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C370" t="str">
         <v/>
@@ -23378,7 +23378,7 @@
         <v>24J-240</v>
       </c>
       <c r="B371" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C371" t="str">
         <v>CITY PNP-TAGBILARAN CITY</v>
@@ -23440,7 +23440,7 @@
         <v>24J-241</v>
       </c>
       <c r="B372" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C372" t="str">
         <v>CITY PNP-TAGBILARAN CITY</v>
@@ -23626,7 +23626,7 @@
         <v>VII-14-INQ-21l-191</v>
       </c>
       <c r="B375" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C375" t="str">
         <v>PNP-TAGBILARAN CITY</v>
@@ -23688,7 +23688,7 @@
         <v>VII-14-INQ-21l-192</v>
       </c>
       <c r="B376" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C376" t="str">
         <v>PNP-TAGBILARAN CITY</v>
@@ -23750,7 +23750,7 @@
         <v>96-1820</v>
       </c>
       <c r="B377" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C377" t="str">
         <v/>
@@ -23812,7 +23812,7 @@
         <v>96-1821</v>
       </c>
       <c r="B378" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C378" t="str">
         <v/>
@@ -23874,7 +23874,7 @@
         <v>96-1822</v>
       </c>
       <c r="B379" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C379" t="str">
         <v/>
@@ -23936,7 +23936,7 @@
         <v>96-772</v>
       </c>
       <c r="B380" t="str">
-        <v>April 10, 2026</v>
+        <v/>
       </c>
       <c r="C380" t="str">
         <v/>

</xml_diff>

<commit_message>
filed in court fixed
</commit_message>
<xml_diff>
--- a/uploads/cases.xlsx
+++ b/uploads/cases.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Cases" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Cases'!A1:T380</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Cases'!A1:T381</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -35,17 +35,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="10">
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
-    <numFmt numFmtId="165" formatCode="m/d/yy"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm"/>
-    <numFmt numFmtId="167" formatCode="yyyy\-m"/>
-    <numFmt numFmtId="168" formatCode="mm/dd/yy"/>
-    <numFmt numFmtId="169" formatCode="mm/yyyy"/>
-    <numFmt numFmtId="170" formatCode="mm\-dd\-yyyy"/>
-    <numFmt numFmtId="171" formatCode="mm/dd"/>
-    <numFmt numFmtId="172" formatCode="m/yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -409,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T380"/>
+  <dimension ref="A1:T381"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -23993,10 +23984,72 @@
         <v>CUTAMORA, FLAVIA_0001.pdf</v>
       </c>
     </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v>Test3</v>
+      </c>
+      <c r="B381" t="str">
+        <v>April 22, 2026</v>
+      </c>
+      <c r="C381" t="str">
+        <v>s</v>
+      </c>
+      <c r="D381" t="str">
+        <v>sdf</v>
+      </c>
+      <c r="E381" t="str">
+        <v>sdfs</v>
+      </c>
+      <c r="F381" t="str">
+        <v>dfsdf</v>
+      </c>
+      <c r="G381" t="str">
+        <v/>
+      </c>
+      <c r="H381" t="str">
+        <v>April 15, 2026</v>
+      </c>
+      <c r="I381" t="str">
+        <v>ada</v>
+      </c>
+      <c r="J381" t="str">
+        <v/>
+      </c>
+      <c r="K381" t="str">
+        <v/>
+      </c>
+      <c r="L381" t="str">
+        <v/>
+      </c>
+      <c r="M381" t="str">
+        <v>zc</v>
+      </c>
+      <c r="N381" t="str">
+        <v>asd</v>
+      </c>
+      <c r="O381" t="str">
+        <v/>
+      </c>
+      <c r="P381" t="str">
+        <v>s</v>
+      </c>
+      <c r="Q381" t="str">
+        <v>Filed in Court</v>
+      </c>
+      <c r="R381" t="str">
+        <v>a</v>
+      </c>
+      <c r="S381" t="str">
+        <v>April 14, 2026</v>
+      </c>
+      <c r="T381" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T380"/>
+  <autoFilter ref="A1:T381"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T380"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T381"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added O.R in format C and add period in No
</commit_message>
<xml_diff>
--- a/uploads/cases.xlsx
+++ b/uploads/cases.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Cases" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Cases'!A1:T383</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Cases'!A1:T380</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T383"/>
+  <dimension ref="A1:T380"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -15805,7 +15805,7 @@
         <v>VII-14-INV 24B-45</v>
       </c>
       <c r="B249" t="str">
-        <v/>
+        <v>February 13, 2024</v>
       </c>
       <c r="C249" t="str">
         <v>TARIAO, ROSALINDA R.</v>
@@ -15867,7 +15867,7 @@
         <v>VII-14-INV 24B-45</v>
       </c>
       <c r="B250" t="str">
-        <v/>
+        <v>February 13, 2024</v>
       </c>
       <c r="C250" t="str">
         <v>TARIAO, ROSALINDA R.</v>
@@ -23984,196 +23984,10 @@
         <v>CUTAMORA, FLAVIA_0001.pdf</v>
       </c>
     </row>
-    <row r="381">
-      <c r="A381" t="str">
-        <v>Test3</v>
-      </c>
-      <c r="B381" t="str">
-        <v>April 21, 2026</v>
-      </c>
-      <c r="C381" t="str">
-        <v>s</v>
-      </c>
-      <c r="D381" t="str">
-        <v>sdf</v>
-      </c>
-      <c r="E381" t="str">
-        <v>sdfs</v>
-      </c>
-      <c r="F381" t="str">
-        <v>dfsdf</v>
-      </c>
-      <c r="G381" t="str">
-        <v/>
-      </c>
-      <c r="H381" t="str">
-        <v>April 14, 2026</v>
-      </c>
-      <c r="I381" t="str">
-        <v>ada</v>
-      </c>
-      <c r="J381" t="str">
-        <v/>
-      </c>
-      <c r="K381" t="str">
-        <v/>
-      </c>
-      <c r="L381" t="str">
-        <v/>
-      </c>
-      <c r="M381" t="str">
-        <v>343dfd</v>
-      </c>
-      <c r="N381" t="str">
-        <v>gdfgdfgdf</v>
-      </c>
-      <c r="O381" t="str">
-        <v/>
-      </c>
-      <c r="P381" t="str">
-        <v>s</v>
-      </c>
-      <c r="Q381" t="str">
-        <v>Filed in Court</v>
-      </c>
-      <c r="R381" t="str">
-        <v>a</v>
-      </c>
-      <c r="S381" t="str">
-        <v>April 13, 2026</v>
-      </c>
-      <c r="T381" t="str">
-        <v>N/A</v>
-      </c>
-    </row>
-    <row r="382">
-      <c r="A382" t="str">
-        <v>Test3</v>
-      </c>
-      <c r="B382" t="str">
-        <v>April 21, 2026</v>
-      </c>
-      <c r="C382" t="str">
-        <v>s</v>
-      </c>
-      <c r="D382" t="str">
-        <v>sdfsfds</v>
-      </c>
-      <c r="E382" t="str">
-        <v>s</v>
-      </c>
-      <c r="F382" t="str">
-        <v>dfsdf</v>
-      </c>
-      <c r="G382" t="str">
-        <v/>
-      </c>
-      <c r="H382" t="str">
-        <v>April 14, 2026</v>
-      </c>
-      <c r="I382" t="str">
-        <v>ada</v>
-      </c>
-      <c r="J382" t="str">
-        <v/>
-      </c>
-      <c r="K382" t="str">
-        <v/>
-      </c>
-      <c r="L382" t="str">
-        <v/>
-      </c>
-      <c r="M382" t="str">
-        <v>sdfsdf</v>
-      </c>
-      <c r="N382" t="str">
-        <v>dfgdfgdfg</v>
-      </c>
-      <c r="O382" t="str">
-        <v/>
-      </c>
-      <c r="P382" t="str">
-        <v>s</v>
-      </c>
-      <c r="Q382" t="str">
-        <v>Pending</v>
-      </c>
-      <c r="R382" t="str">
-        <v>a</v>
-      </c>
-      <c r="S382" t="str">
-        <v>April 13, 2026</v>
-      </c>
-      <c r="T382" t="str">
-        <v>N/A</v>
-      </c>
-    </row>
-    <row r="383">
-      <c r="A383" t="str">
-        <v>Test3</v>
-      </c>
-      <c r="B383" t="str">
-        <v>April 21, 2026</v>
-      </c>
-      <c r="C383" t="str">
-        <v>s</v>
-      </c>
-      <c r="D383" t="str">
-        <v>sdfsdfsdf</v>
-      </c>
-      <c r="E383" t="str">
-        <v>s</v>
-      </c>
-      <c r="F383" t="str">
-        <v>dfsdf</v>
-      </c>
-      <c r="G383" t="str">
-        <v/>
-      </c>
-      <c r="H383" t="str">
-        <v>April 14, 2026</v>
-      </c>
-      <c r="I383" t="str">
-        <v>ada</v>
-      </c>
-      <c r="J383" t="str">
-        <v/>
-      </c>
-      <c r="K383" t="str">
-        <v/>
-      </c>
-      <c r="L383" t="str">
-        <v/>
-      </c>
-      <c r="M383" t="str">
-        <v>dfgdfgdfg</v>
-      </c>
-      <c r="N383" t="str">
-        <v>sdf</v>
-      </c>
-      <c r="O383" t="str">
-        <v/>
-      </c>
-      <c r="P383" t="str">
-        <v>sdfsdfs</v>
-      </c>
-      <c r="Q383" t="str">
-        <v>Pending</v>
-      </c>
-      <c r="R383" t="str">
-        <v>a</v>
-      </c>
-      <c r="S383" t="str">
-        <v>April 13, 2026</v>
-      </c>
-      <c r="T383" t="str">
-        <v>N/A</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:T383"/>
+  <autoFilter ref="A1:T380"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T383"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T380"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>